<commit_message>
traffic-triage-eval: status optional, AWS WAF labels, harmless-split rule
- `status` is no longer required: WAF logs carry the verdict, not the
  backend's answer. The profile drops the 404-rate signals and says why;
  questions fall back to volume and WAF verdicts.
- New optional `waf_labels` (AWS WAF `labels[].name`): attack-signature,
  bot-control and IP-reputation labels become code signals and count as
  payload evidence for the attack floor.
- Schema doc: AWS WAF field mapping verified against the log-field
  reference (RATE_BASED -> throttle, COUNT matches, responseCodeSent,
  httpSourceName, headers[] for Host / UA / Referer).
- A low-confidence choice split between benign_user and benign_bot keeps
  the top label instead of becoming unclear.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QaG5kHPxSosfJfLwgjAgJQ
</commit_message>
<xml_diff>
--- a/skills/jev/traffic-triage-eval/mock-data/example-output/results.xlsx
+++ b/skills/jev/traffic-triage-eval/mock-data/example-output/results.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read me" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$Q$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Results'!$A$1:$R$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Details'!$A$1:$Z$34</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -462,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q34"/>
+  <dimension ref="A1:R34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -475,13 +475,14 @@
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="44" customWidth="1" min="11" max="11"/>
-    <col width="56" customWidth="1" min="12" max="12"/>
-    <col width="50" customWidth="1" min="13" max="13"/>
-    <col width="8" customWidth="1" min="14" max="14"/>
-    <col width="30" customWidth="1" min="15" max="15"/>
-    <col width="70" customWidth="1" min="16" max="16"/>
-    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
+    <col width="44" customWidth="1" min="12" max="12"/>
+    <col width="56" customWidth="1" min="13" max="13"/>
+    <col width="50" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+    <col width="70" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -537,35 +538,40 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
+          <t>WAF labels</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Signals (Jev)</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Code signals</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Top UA</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>ASN</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Hosts</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Sample paths</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
@@ -583,7 +589,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2.82</v>
+        <v>2.79</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -610,37 +616,38 @@
       <c r="J2" t="n">
         <v>19</v>
       </c>
-      <c r="K2" s="3" t="inlineStr">
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>exploit_payloads, app_aware, automated, enumeration</t>
         </is>
       </c>
-      <c r="L2" s="3" t="inlineStr">
+      <c r="M2" s="3" t="inlineStr">
         <is>
           <t>payloads: 55 requests with exploit-shaped strings: sqli=29, xss=26; waf_denied: 19 requests denied by the WAF; enumeration: 8 distinct ids under /api/v1/trust/documents?tenant_id=</t>
         </is>
       </c>
-      <c r="M2" s="3" t="inlineStr">
+      <c r="N2" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 (Macintosh; Intel Mac OS X 14_5) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/128.0.0.0 Safari/537.36</t>
         </is>
       </c>
-      <c r="N2" t="n">
+      <c r="O2" t="n">
         <v>49505</v>
       </c>
-      <c r="O2" s="3" t="inlineStr">
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io, trust.example-trust.io</t>
         </is>
       </c>
-      <c r="P2" s="3" t="inlineStr">
+      <c r="Q2" s="3" t="inlineStr">
         <is>
           <t>22x /api/v1/trust/documents [403/200]
 20x /api/v1/tenants/acme/documents [200/400]
 18x /acme/documents [400/200]</t>
         </is>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="R2" t="inlineStr">
         <is>
           <t>malicious</t>
         </is>
@@ -658,7 +665,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2.78</v>
+        <v>2.79</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -685,30 +692,31 @@
       <c r="J3" t="n">
         <v>0</v>
       </c>
-      <c r="K3" s="3" t="inlineStr">
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" s="3" t="inlineStr">
         <is>
           <t>exploit_payloads, app_aware, automated</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>ua_script: 22 of 30 requests carry a script-class User-Agent; payloads: 40 requests with exploit-shaped strings: ssrf=25, template_injection=5, log4shell_jndi=5, scanner_marker=5</t>
         </is>
       </c>
-      <c r="M3" s="3" t="inlineStr">
+      <c r="N3" s="3" t="inlineStr">
         <is>
           <t>python-requests/2.31.0</t>
         </is>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>209588</v>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P3" s="3" t="inlineStr">
+      <c r="Q3" s="3" t="inlineStr">
         <is>
           <t>11x /api/v1/tenants/acme/documents/preview [403/400]
 10x /api/v1/tenants/acme/pages/import [400/401]
@@ -716,7 +724,7 @@
 4x /api/v1/tenants/acme/settings [401/403]</t>
         </is>
       </c>
-      <c r="Q3" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>malicious</t>
         </is>
@@ -734,7 +742,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2.77</v>
+        <v>2.74</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -761,30 +769,31 @@
       <c r="J4" t="n">
         <v>0</v>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>exploit_payloads, app_aware, automated</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>ua_script: 24 of 24 requests carry a script-class User-Agent; payloads: 24 requests with exploit-shaped strings: deserialization=13, template_injection=11</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>Apache-HttpClient/4.5.14 (Java/17.0.2)</t>
         </is>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>47583</v>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>10x /api/v1/tenants/acme/members [400/401]
 6x /api/v1/tenants/acme/settings [400/401]
@@ -792,7 +801,7 @@
 3x /api/v1/tenants/acme/documents [401]</t>
         </is>
       </c>
-      <c r="Q4" t="inlineStr">
+      <c r="R4" t="inlineStr">
         <is>
           <t>malicious</t>
         </is>
@@ -810,7 +819,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2.52</v>
+        <v>2.48</v>
       </c>
       <c r="D5" t="n">
         <v>0.97</v>
@@ -837,35 +846,36 @@
       <c r="J5" t="n">
         <v>0</v>
       </c>
-      <c r="K5" s="3" t="inlineStr">
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" s="3" t="inlineStr">
         <is>
           <t>credential_attack, app_aware, automated</t>
         </is>
       </c>
-      <c r="L5" s="3" t="inlineStr">
+      <c r="M5" s="3" t="inlineStr">
         <is>
           <t>ua_script: 200 of 200 requests carry a script-class User-Agent; waf_throttled: 190 requests rate-limited by the WAF; auth_volume: 200 requests to authentication endpoints</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
+      <c r="N5" s="3" t="inlineStr">
         <is>
           <t>axios/1.7.2</t>
         </is>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>63949</v>
       </c>
-      <c r="O5" s="3" t="inlineStr">
+      <c r="P5" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P5" s="3" t="inlineStr">
+      <c r="Q5" s="3" t="inlineStr">
         <is>
           <t>200x /api/v1/auth/oauth/register [429/201]</t>
         </is>
       </c>
-      <c r="Q5" t="inlineStr">
+      <c r="R5" t="inlineStr">
         <is>
           <t>malicious</t>
         </is>
@@ -883,7 +893,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2.34</v>
+        <v>2.32</v>
       </c>
       <c r="D6" t="n">
         <v>0.99</v>
@@ -910,30 +920,31 @@
       <c r="J6" t="n">
         <v>8</v>
       </c>
-      <c r="K6" s="3" t="inlineStr">
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" s="3" t="inlineStr">
         <is>
           <t>exploit_payloads, app_aware, generic_probing, automated</t>
         </is>
       </c>
-      <c r="L6" s="3" t="inlineStr">
+      <c r="M6" s="3" t="inlineStr">
         <is>
           <t>payloads: 20 requests with exploit-shaped strings: traversal=20; waf_denied: 8 requests denied by the WAF</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
+      <c r="N6" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 (Macintosh; Intel Mac OS X 14_5) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/128.0.0.0 Safari/537.36</t>
         </is>
       </c>
-      <c r="N6" t="n">
+      <c r="O6" t="n">
         <v>209605</v>
       </c>
-      <c r="O6" s="3" t="inlineStr">
+      <c r="P6" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P6" s="3" t="inlineStr">
+      <c r="Q6" s="3" t="inlineStr">
         <is>
           <t>4x /api/v1/tenants/acme/documents/../../../../etc/passwd [400/404]
 4x /assets/..%2f..%2f.env [400/403]
@@ -942,7 +953,7 @@
 4x /acme/documents/....//....//etc/shadow [400/403]</t>
         </is>
       </c>
-      <c r="Q6" t="inlineStr">
+      <c r="R6" t="inlineStr">
         <is>
           <t>malicious</t>
         </is>
@@ -960,7 +971,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2.23</v>
+        <v>2.28</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -987,30 +998,31 @@
       <c r="J7" t="n">
         <v>14</v>
       </c>
-      <c r="K7" s="3" t="inlineStr">
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" s="3" t="inlineStr">
         <is>
           <t>exploit_payloads, automated, scanner_tool, app_aware, credential_attack</t>
         </is>
       </c>
-      <c r="L7" s="3" t="inlineStr">
+      <c r="M7" s="3" t="inlineStr">
         <is>
           <t>ua_scanner: 140 of 140 requests carry a scanner-class User-Agent; payloads: 53 requests with exploit-shaped strings: template_injection=19, scanner_marker=19, traversal=15; waf_denied: 14 requests denied by the WAF; burst: peak 140 requests in one minute</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
+      <c r="N7" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 (Nuclei - Open-source project (github.com/projectdiscovery/nuclei))</t>
         </is>
       </c>
-      <c r="N7" t="n">
+      <c r="O7" t="n">
         <v>396507</v>
       </c>
-      <c r="O7" s="3" t="inlineStr">
+      <c r="P7" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P7" s="3" t="inlineStr">
+      <c r="Q7" s="3" t="inlineStr">
         <is>
           <t>42x /api/v1/tenants/acme/documents [400/405]
 32x /api/v1/auth/user_info [405/400]
@@ -1020,7 +1032,7 @@
 15x /api/v1/tenants/acme/audit [404/401]</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
+      <c r="R7" t="inlineStr">
         <is>
           <t>malicious</t>
         </is>
@@ -1038,130 +1050,58 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2.18</v>
+        <v>2.15</v>
       </c>
       <c r="D8" t="n">
+        <v>0.72</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>89.248.165.2</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>46</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>01:44-09:29 (464.9 min)</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
         <v>1</v>
       </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>5.188.86.2</t>
-        </is>
-      </c>
-      <c r="F8" t="n">
-        <v>420</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>02:50-02:51 (1.8 min)</t>
-        </is>
-      </c>
-      <c r="H8" t="n">
-        <v>239</v>
-      </c>
       <c r="I8" t="n">
-        <v>0</v>
+        <v>0.78</v>
       </c>
       <c r="J8" t="n">
         <v>0</v>
       </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>credential_attack, app_aware, automated</t>
-        </is>
-      </c>
+      <c r="K8" t="inlineStr"/>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>waf_throttled: 254 requests rate-limited by the WAF; auth_volume: 420 requests to authentication endpoints; burst: peak 239 requests in one minute</t>
+          <t>app_aware, enumeration</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>Mozilla/5.0 (Windows NT 10.0; Win64; x64) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/124.0.0.0 Safari/537.36</t>
-        </is>
-      </c>
-      <c r="N8" t="n">
-        <v>34665</v>
-      </c>
-      <c r="O8" s="3" t="inlineStr">
-        <is>
-          <t>app.example-trust.io</t>
-        </is>
+          <t>enumeration: 40 distinct ids under /api/v1/trust/documents/{uuid}</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>Mozilla/5.0 (Windows NT 10.0; Win64; x64; rv:130.0) Gecko/20100101 Firefox/130.0</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>202425</v>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>420x /api/v1/auth/signin-password [429/401]</t>
-        </is>
-      </c>
-      <c r="Q8" t="inlineStr">
-        <is>
-          <t>malicious</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>malicious</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>2.16</v>
-      </c>
-      <c r="D9" t="n">
-        <v>0.77</v>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>89.248.165.2</t>
-        </is>
-      </c>
-      <c r="F9" t="n">
-        <v>46</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>01:44-09:29 (464.9 min)</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>1</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-      <c r="K9" s="3" t="inlineStr">
-        <is>
-          <t>app_aware, enumeration</t>
-        </is>
-      </c>
-      <c r="L9" s="3" t="inlineStr">
-        <is>
-          <t>enumeration: 40 distinct ids under /api/v1/trust/documents/{uuid}</t>
-        </is>
-      </c>
-      <c r="M9" s="3" t="inlineStr">
-        <is>
-          <t>Mozilla/5.0 (Windows NT 10.0; Win64; x64; rv:130.0) Gecko/20100101 Firefox/130.0</t>
-        </is>
-      </c>
-      <c r="N9" t="n">
-        <v>202425</v>
-      </c>
-      <c r="O9" s="3" t="inlineStr">
-        <is>
           <t>trust.example-trust.io, app.example-trust.io</t>
         </is>
       </c>
-      <c r="P9" s="3" t="inlineStr">
+      <c r="Q8" s="3" t="inlineStr">
         <is>
           <t>1x / [200]
 1x /api/v1/auth/user_info [401]
@@ -1173,7 +1113,81 @@
 1x /api/v1/trust/documents/8ff19886-d5bf-4926-ad84-0689ceed0ffc [404]</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>malicious</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>malicious</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>2.14</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>5.188.86.2</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>420</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>02:50-02:51 (1.8 min)</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>239</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" s="3" t="inlineStr">
+        <is>
+          <t>credential_attack, app_aware, automated</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>waf_throttled: 254 requests rate-limited by the WAF; auth_volume: 420 requests to authentication endpoints; burst: peak 239 requests in one minute</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>Mozilla/5.0 (Windows NT 10.0; Win64; x64) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/124.0.0.0 Safari/537.36</t>
+        </is>
+      </c>
+      <c r="O9" t="n">
+        <v>34665</v>
+      </c>
+      <c r="P9" s="3" t="inlineStr">
+        <is>
+          <t>app.example-trust.io</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>420x /api/v1/auth/signin-password [429/401]</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
         <is>
           <t>malicious</t>
         </is>
@@ -1191,7 +1205,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2.09</v>
+        <v>2.12</v>
       </c>
       <c r="D10" t="n">
         <v>0.99</v>
@@ -1218,35 +1232,36 @@
       <c r="J10" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>automated, app_aware, enumeration</t>
-        </is>
-      </c>
+      <c r="K10" t="inlineStr"/>
       <c r="L10" s="3" t="inlineStr">
         <is>
+          <t>automated, enumeration, app_aware</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr">
+        <is>
           <t>ua_script: 300 of 300 requests carry a script-class User-Agent; enumeration: 300 distinct ids under /api/v1/trust/pages?tenant_id=</t>
         </is>
       </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="N10" s="3" t="inlineStr">
         <is>
           <t>okhttp/4.12.0</t>
         </is>
       </c>
-      <c r="N10" t="n">
+      <c r="O10" t="n">
         <v>136787</v>
       </c>
-      <c r="O10" s="3" t="inlineStr">
+      <c r="P10" s="3" t="inlineStr">
         <is>
           <t>trust.example-trust.io</t>
         </is>
       </c>
-      <c r="P10" s="3" t="inlineStr">
+      <c r="Q10" s="3" t="inlineStr">
         <is>
           <t>300x /api/v1/trust/pages [404/200]</t>
         </is>
       </c>
-      <c r="Q10" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>malicious</t>
         </is>
@@ -1263,7 +1278,7 @@
         <v>1.06</v>
       </c>
       <c r="D11" t="n">
-        <v>0.78</v>
+        <v>0.8</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -1287,36 +1302,37 @@
       <c r="J11" t="n">
         <v>0</v>
       </c>
-      <c r="K11" s="3" t="inlineStr">
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" s="3" t="inlineStr">
         <is>
           <t>wrong_host, automated, scanner_tool</t>
         </is>
       </c>
-      <c r="L11" s="3" t="inlineStr">
+      <c r="M11" s="3" t="inlineStr">
         <is>
           <t>ua_scanner: 2 of 2 requests carry a scanner-class User-Agent; raw_ip_host: 2 requests addressed the server by IP instead of a hostname</t>
         </is>
       </c>
-      <c r="M11" s="3" t="inlineStr">
+      <c r="N11" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 zgrab/0.x</t>
         </is>
       </c>
-      <c r="N11" t="n">
+      <c r="O11" t="n">
         <v>398324</v>
       </c>
-      <c r="O11" s="3" t="inlineStr">
+      <c r="P11" s="3" t="inlineStr">
         <is>
           <t>203.0.113.200</t>
         </is>
       </c>
-      <c r="P11" s="3" t="inlineStr">
+      <c r="Q11" s="3" t="inlineStr">
         <is>
           <t>1x / [200]
 1x /robots.txt [404]</t>
         </is>
       </c>
-      <c r="Q11" t="inlineStr">
+      <c r="R11" t="inlineStr">
         <is>
           <t>background_scan</t>
         </is>
@@ -1330,126 +1346,58 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.03</v>
+        <v>1.01</v>
       </c>
       <c r="D12" t="n">
-        <v>0.5</v>
+        <v>0.95</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>87.120.104.29</t>
+          <t>80.94.95.211</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>22:00-22:29 (29.0 min)</t>
+          <t>21:15-21:15 (0.1 min)</t>
         </is>
       </c>
       <c r="H12" t="n">
+        <v>45</v>
+      </c>
+      <c r="I12" t="n">
         <v>1</v>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>0</v>
       </c>
-      <c r="J12" t="n">
-        <v>30</v>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>wrong_host, automated</t>
-        </is>
-      </c>
+      <c r="K12" t="inlineStr"/>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>waf_denied: 30 requests denied by the WAF</t>
+          <t>generic_probing, automated, scanner_tool</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>Mozilla/5.0 (Linux; Android 10) AppleWebKit/537.36</t>
-        </is>
-      </c>
-      <c r="N12" t="n">
-        <v>34224</v>
-      </c>
-      <c r="O12" s="3" t="inlineStr">
-        <is>
-          <t>vwnfnjosqnhsomoqaqsn.example-cdn.net</t>
-        </is>
+          <t>ua_scanner: 45 of 45 requests carry a scanner-class User-Agent; probe_paths: 45 requests for 1 scanner path families: backup_files=45</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>Go-http-client/1.1</t>
+        </is>
+      </c>
+      <c r="O12" t="n">
+        <v>204428</v>
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
-          <t>30x / [502]</t>
-        </is>
-      </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>background_scan</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>background_scan</t>
-        </is>
-      </c>
-      <c r="C13" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="D13" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>80.94.95.211</t>
-        </is>
-      </c>
-      <c r="F13" t="n">
-        <v>45</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>21:15-21:15 (0.1 min)</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>45</v>
-      </c>
-      <c r="I13" t="n">
-        <v>1</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>generic_probing, automated, scanner_tool</t>
-        </is>
-      </c>
-      <c r="L13" s="3" t="inlineStr">
-        <is>
-          <t>ua_scanner: 45 of 45 requests carry a scanner-class User-Agent; probe_paths: 45 requests for 1 scanner path families: backup_files=45</t>
-        </is>
-      </c>
-      <c r="M13" s="3" t="inlineStr">
-        <is>
-          <t>Go-http-client/1.1</t>
-        </is>
-      </c>
-      <c r="N13" t="n">
-        <v>204428</v>
-      </c>
-      <c r="O13" s="3" t="inlineStr">
-        <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P13" s="3" t="inlineStr">
+      <c r="Q12" s="3" t="inlineStr">
         <is>
           <t>1x /backup.zip [404]
 1x /backup.sql [404]
@@ -1461,7 +1409,77 @@
 1x /site.tar.gz [404]</t>
         </is>
       </c>
-      <c r="Q13" t="inlineStr">
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>background_scan</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>background_scan</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>87.120.104.29</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>30</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>22:00-22:29 (29.0 min)</t>
+        </is>
+      </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>30</v>
+      </c>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>wrong_host, automated</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr">
+        <is>
+          <t>waf_denied: 30 requests denied by the WAF</t>
+        </is>
+      </c>
+      <c r="N13" s="3" t="inlineStr">
+        <is>
+          <t>Mozilla/5.0 (Linux; Android 10) AppleWebKit/537.36</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>34224</v>
+      </c>
+      <c r="P13" s="3" t="inlineStr">
+        <is>
+          <t>vwnfnjosqnhsomoqaqsn.example-cdn.net</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>30x / [502]</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
         <is>
           <t>background_scan</t>
         </is>
@@ -1502,30 +1520,31 @@
       <c r="J14" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="3" t="inlineStr">
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" s="3" t="inlineStr">
         <is>
           <t>generic_probing, automated, wrong_host, scanner_tool</t>
         </is>
       </c>
-      <c r="L14" s="3" t="inlineStr">
+      <c r="M14" s="3" t="inlineStr">
         <is>
           <t>ua_script: 27 of 27 requests carry a script-class User-Agent; probe_paths: 24 requests for 1 scanner path families: php_admin=24; raw_ip_host: 27 requests addressed the server by IP instead of a hostname</t>
         </is>
       </c>
-      <c r="M14" s="3" t="inlineStr">
+      <c r="N14" s="3" t="inlineStr">
         <is>
           <t>python-requests/2.28.1</t>
         </is>
       </c>
-      <c r="N14" t="n">
+      <c r="O14" t="n">
         <v>394711</v>
       </c>
-      <c r="O14" s="3" t="inlineStr">
+      <c r="P14" s="3" t="inlineStr">
         <is>
           <t>203.0.113.200</t>
         </is>
       </c>
-      <c r="P14" s="3" t="inlineStr">
+      <c r="Q14" s="3" t="inlineStr">
         <is>
           <t>3x /phpmyadmin/index.php [404]
 3x /pma/index.php [404]
@@ -1537,7 +1556,7 @@
 3x /sql/ [404]</t>
         </is>
       </c>
-      <c r="Q14" t="inlineStr">
+      <c r="R14" t="inlineStr">
         <is>
           <t>background_scan</t>
         </is>
@@ -1578,30 +1597,31 @@
       <c r="J15" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="3" t="inlineStr">
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr">
         <is>
           <t>generic_probing, wrong_host, automated, scanner_tool</t>
         </is>
       </c>
-      <c r="L15" s="3" t="inlineStr">
+      <c r="M15" s="3" t="inlineStr">
         <is>
           <t>probe_paths: 26 requests for 3 scanner path families: wordpress=14, php_admin=8, env_files=4; raw_ip_host: 18 requests addressed the server by IP instead of a hostname</t>
         </is>
       </c>
-      <c r="M15" s="3" t="inlineStr">
+      <c r="N15" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 (Windows NT 10.0; Win64; x64) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/91.0.4472.124 Safari/537.36</t>
         </is>
       </c>
-      <c r="N15" t="n">
+      <c r="O15" t="n">
         <v>44477</v>
       </c>
-      <c r="O15" s="3" t="inlineStr">
+      <c r="P15" s="3" t="inlineStr">
         <is>
           <t>203.0.113.200</t>
         </is>
       </c>
-      <c r="P15" s="3" t="inlineStr">
+      <c r="Q15" s="3" t="inlineStr">
         <is>
           <t>2x /wp-login.php [404]
 2x /xmlrpc.php [404]
@@ -1613,7 +1633,7 @@
 2x /wordpress/wp-login.php [404]</t>
         </is>
       </c>
-      <c r="Q15" t="inlineStr">
+      <c r="R15" t="inlineStr">
         <is>
           <t>background_scan</t>
         </is>
@@ -1654,30 +1674,31 @@
       <c r="J16" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="3" t="inlineStr">
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr">
         <is>
           <t>generic_probing, wrong_host, automated, scanner_tool</t>
         </is>
       </c>
-      <c r="L16" s="3" t="inlineStr">
+      <c r="M16" s="3" t="inlineStr">
         <is>
           <t>ua_empty: 7 of 7 requests carry a empty-class User-Agent; probe_paths: 6 requests for 1 scanner path families: shells_exploits=6; raw_ip_host: 7 requests addressed the server by IP instead of a hostname</t>
         </is>
       </c>
-      <c r="M16" s="3" t="inlineStr">
+      <c r="N16" s="3" t="inlineStr">
         <is>
           <t>(empty)</t>
         </is>
       </c>
-      <c r="N16" t="n">
+      <c r="O16" t="n">
         <v>202425</v>
       </c>
-      <c r="O16" s="3" t="inlineStr">
+      <c r="P16" s="3" t="inlineStr">
         <is>
           <t>203.0.113.200</t>
         </is>
       </c>
-      <c r="P16" s="3" t="inlineStr">
+      <c r="Q16" s="3" t="inlineStr">
         <is>
           <t>1x /cgi-bin/luci [404]
 1x /setup.cgi [404]
@@ -1688,7 +1709,7 @@
 1x /shell [404]</t>
         </is>
       </c>
-      <c r="Q16" t="inlineStr">
+      <c r="R16" t="inlineStr">
         <is>
           <t>background_scan</t>
         </is>
@@ -1702,10 +1723,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.49</v>
       </c>
       <c r="D17" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -1729,37 +1750,38 @@
       <c r="J17" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="3" t="inlineStr">
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" s="3" t="inlineStr">
         <is>
           <t>wrong_host, automated, scanner_tool, declared_bot</t>
         </is>
       </c>
-      <c r="L17" s="3" t="inlineStr">
+      <c r="M17" s="3" t="inlineStr">
         <is>
           <t>ua_scanner: 3 of 3 requests carry a scanner-class User-Agent; raw_ip_host: 3 requests addressed the server by IP instead of a hostname</t>
         </is>
       </c>
-      <c r="M17" s="3" t="inlineStr">
+      <c r="N17" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 (compatible; CensysInspect/1.1; +https://about.censys.io/)</t>
         </is>
       </c>
-      <c r="N17" t="n">
+      <c r="O17" t="n">
         <v>398324</v>
       </c>
-      <c r="O17" s="3" t="inlineStr">
+      <c r="P17" s="3" t="inlineStr">
         <is>
           <t>203.0.113.200</t>
         </is>
       </c>
-      <c r="P17" s="3" t="inlineStr">
+      <c r="Q17" s="3" t="inlineStr">
         <is>
           <t>1x /robots.txt [404]
 1x / [200]
 1x /.well-known/security.txt [404]</t>
         </is>
       </c>
-      <c r="Q17" t="inlineStr">
+      <c r="R17" t="inlineStr">
         <is>
           <t>background_scan</t>
         </is>
@@ -1773,10 +1795,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.7</v>
+        <v>0.74</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -1800,30 +1822,31 @@
       <c r="J18" t="n">
         <v>0</v>
       </c>
-      <c r="K18" s="3" t="inlineStr">
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" s="3" t="inlineStr">
         <is>
           <t>ai_operated, app_aware, automated</t>
         </is>
       </c>
-      <c r="L18" s="3" t="inlineStr">
+      <c r="M18" s="3" t="inlineStr">
         <is>
           <t>ua_ai_agent: 4 of 4 requests carry a ai_agent-class User-Agent</t>
         </is>
       </c>
-      <c r="M18" s="3" t="inlineStr">
+      <c r="N18" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 (X11; Linux x86_64) AppleWebKit/537.36 (KHTML, like Gecko) HeadlessChrome/128.0.0.0 Safari/537.36 browser-use/0.3</t>
         </is>
       </c>
-      <c r="N18" t="n">
+      <c r="O18" t="n">
         <v>15169</v>
       </c>
-      <c r="O18" s="3" t="inlineStr">
+      <c r="P18" s="3" t="inlineStr">
         <is>
           <t>trust.example-trust.io</t>
         </is>
       </c>
-      <c r="P18" s="3" t="inlineStr">
+      <c r="Q18" s="3" t="inlineStr">
         <is>
           <t>1x /acme [200]
 1x /acme/documents [200]
@@ -1831,7 +1854,7 @@
 1x /acme/faq [200]</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
+      <c r="R18" t="inlineStr">
         <is>
           <t>ai_agent</t>
         </is>
@@ -1845,7 +1868,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.64</v>
+        <v>0.71</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
@@ -1872,30 +1895,31 @@
       <c r="J19" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="3" t="inlineStr">
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" s="3" t="inlineStr">
         <is>
           <t>ai_operated, app_aware, automated, declared_bot</t>
         </is>
       </c>
-      <c r="L19" s="3" t="inlineStr">
+      <c r="M19" s="3" t="inlineStr">
         <is>
           <t>ua_ai_agent: 21 of 21 requests carry a ai_agent-class User-Agent</t>
         </is>
       </c>
-      <c r="M19" s="3" t="inlineStr">
+      <c r="N19" s="3" t="inlineStr">
         <is>
           <t>mcp-client/1.0 (claude-desktop; model-context-protocol)</t>
         </is>
       </c>
-      <c r="N19" t="n">
+      <c r="O19" t="n">
         <v>14618</v>
       </c>
-      <c r="O19" s="3" t="inlineStr">
+      <c r="P19" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P19" s="3" t="inlineStr">
+      <c r="Q19" s="3" t="inlineStr">
         <is>
           <t>18x /mcp [200]
 1x /api/v1/auth/oauth/register [201]
@@ -1903,7 +1927,7 @@
 1x /api/v1/auth/oauth/token [200]</t>
         </is>
       </c>
-      <c r="Q19" t="inlineStr">
+      <c r="R19" t="inlineStr">
         <is>
           <t>ai_agent</t>
         </is>
@@ -1917,22 +1941,22 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.58</v>
+        <v>0.49</v>
       </c>
       <c r="D20" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>3.15.8.8</t>
+          <t>20.171.207.1</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>10:00-12:48 (168.0 min)</t>
+          <t>06:00-09:57 (237.0 min)</t>
         </is>
       </c>
       <c r="H20" t="n">
@@ -1944,102 +1968,31 @@
       <c r="J20" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="3" t="inlineStr">
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" s="3" t="inlineStr">
         <is>
           <t>ai_operated, app_aware, automated, declared_bot</t>
         </is>
       </c>
-      <c r="L20" s="3" t="inlineStr">
-        <is>
-          <t>ua_ai_agent: 25 of 25 requests carry a ai_agent-class User-Agent</t>
-        </is>
-      </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>Mozilla/5.0 AppleWebKit/537.36 (KHTML, like Gecko; compatible; PerplexityBot/1.0; +https://perplexity.ai/perplexitybot)</t>
-        </is>
-      </c>
-      <c r="N20" t="n">
-        <v>16509</v>
-      </c>
-      <c r="O20" s="3" t="inlineStr">
+          <t>ua_ai_agent: 80 of 80 requests carry a ai_agent-class User-Agent</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t>Mozilla/5.0 AppleWebKit/537.36 (KHTML, like Gecko; compatible; GPTBot/1.2; +https://openai.com/gptbot)</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>8075</v>
+      </c>
+      <c r="P20" s="3" t="inlineStr">
         <is>
           <t>trust.example-trust.io</t>
         </is>
       </c>
-      <c r="P20" s="3" t="inlineStr">
-        <is>
-          <t>9x /api/v1/trust/pages [200]
-7x /acme/documents [200]
-5x /api/v1/trust/documents [200]
-4x /acme [200]</t>
-        </is>
-      </c>
-      <c r="Q20" t="inlineStr">
-        <is>
-          <t>ai_agent</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" s="5" t="inlineStr">
-        <is>
-          <t>ai_agent</t>
-        </is>
-      </c>
-      <c r="C21" t="n">
-        <v>0.51</v>
-      </c>
-      <c r="D21" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>20.171.207.1</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>80</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>06:00-09:57 (237.0 min)</t>
-        </is>
-      </c>
-      <c r="H21" t="n">
-        <v>1</v>
-      </c>
-      <c r="I21" t="n">
-        <v>0</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="3" t="inlineStr">
-        <is>
-          <t>ai_operated, app_aware, automated, declared_bot</t>
-        </is>
-      </c>
-      <c r="L21" s="3" t="inlineStr">
-        <is>
-          <t>ua_ai_agent: 80 of 80 requests carry a ai_agent-class User-Agent</t>
-        </is>
-      </c>
-      <c r="M21" s="3" t="inlineStr">
-        <is>
-          <t>Mozilla/5.0 AppleWebKit/537.36 (KHTML, like Gecko; compatible; GPTBot/1.2; +https://openai.com/gptbot)</t>
-        </is>
-      </c>
-      <c r="N21" t="n">
-        <v>8075</v>
-      </c>
-      <c r="O21" s="3" t="inlineStr">
-        <is>
-          <t>trust.example-trust.io</t>
-        </is>
-      </c>
-      <c r="P21" s="3" t="inlineStr">
+      <c r="Q20" s="3" t="inlineStr">
         <is>
           <t>21x /acme/faq [200]
 17x /acme/documents [200]
@@ -2048,7 +2001,80 @@
 13x /api/v1/trust/documents [200]</t>
         </is>
       </c>
-      <c r="Q21" t="inlineStr">
+      <c r="R20" t="inlineStr">
+        <is>
+          <t>ai_agent</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>ai_agent</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>3.15.8.8</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>25</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>10:00-12:48 (168.0 min)</t>
+        </is>
+      </c>
+      <c r="H21" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0</v>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>ai_operated, app_aware, automated, declared_bot</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr">
+        <is>
+          <t>ua_ai_agent: 25 of 25 requests carry a ai_agent-class User-Agent</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="inlineStr">
+        <is>
+          <t>Mozilla/5.0 AppleWebKit/537.36 (KHTML, like Gecko; compatible; PerplexityBot/1.0; +https://perplexity.ai/perplexitybot)</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>16509</v>
+      </c>
+      <c r="P21" s="3" t="inlineStr">
+        <is>
+          <t>trust.example-trust.io</t>
+        </is>
+      </c>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>9x /api/v1/trust/pages [200]
+7x /acme/documents [200]
+5x /api/v1/trust/documents [200]
+4x /acme [200]</t>
+        </is>
+      </c>
+      <c r="R21" t="inlineStr">
         <is>
           <t>ai_agent</t>
         </is>
@@ -2062,7 +2088,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.37</v>
+        <v>0.4</v>
       </c>
       <c r="D22" t="n">
         <v>0.99</v>
@@ -2089,30 +2115,31 @@
       <c r="J22" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="3" t="inlineStr">
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" s="3" t="inlineStr">
         <is>
           <t>ai_operated, app_aware, automated, declared_bot</t>
         </is>
       </c>
-      <c r="L22" s="3" t="inlineStr">
+      <c r="M22" s="3" t="inlineStr">
         <is>
           <t>ua_ai_agent: 40 of 40 requests carry a ai_agent-class User-Agent</t>
         </is>
       </c>
-      <c r="M22" s="3" t="inlineStr">
+      <c r="N22" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 AppleWebKit/537.36 (KHTML, like Gecko; compatible; ClaudeBot/1.0; +claudebot@anthropic.com)</t>
         </is>
       </c>
-      <c r="N22" t="n">
+      <c r="O22" t="n">
         <v>16509</v>
       </c>
-      <c r="O22" s="3" t="inlineStr">
+      <c r="P22" s="3" t="inlineStr">
         <is>
           <t>trust.example-trust.io</t>
         </is>
       </c>
-      <c r="P22" s="3" t="inlineStr">
+      <c r="Q22" s="3" t="inlineStr">
         <is>
           <t>9x /api/v1/trust/pages [200]
 9x /acme/documents [200]
@@ -2121,7 +2148,7 @@
 6x /acme [200]</t>
         </is>
       </c>
-      <c r="Q22" t="inlineStr">
+      <c r="R22" t="inlineStr">
         <is>
           <t>ai_agent</t>
         </is>
@@ -2135,10 +2162,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.92</v>
+        <v>0.71</v>
       </c>
       <c r="D23" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -2162,35 +2189,36 @@
       <c r="J23" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="3" t="inlineStr">
-        <is>
-          <t>app_aware, automated, monitoring</t>
-        </is>
-      </c>
+      <c r="K23" t="inlineStr"/>
       <c r="L23" s="3" t="inlineStr">
         <is>
+          <t>automated, app_aware, monitoring</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr">
+        <is>
           <t>ua_script: 96 of 96 requests carry a script-class User-Agent</t>
         </is>
       </c>
-      <c r="M23" s="3" t="inlineStr">
+      <c r="N23" s="3" t="inlineStr">
         <is>
           <t>python-requests/2.32.3</t>
         </is>
       </c>
-      <c r="N23" t="n">
+      <c r="O23" t="n">
         <v>16509</v>
       </c>
-      <c r="O23" s="3" t="inlineStr">
+      <c r="P23" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P23" s="3" t="inlineStr">
+      <c r="Q23" s="3" t="inlineStr">
         <is>
           <t>96x /api/v1/tenants/acme/documents [200]</t>
         </is>
       </c>
-      <c r="Q23" t="inlineStr">
+      <c r="R23" t="inlineStr">
         <is>
           <t>benign_bot</t>
         </is>
@@ -2204,10 +2232,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.65</v>
+        <v>0.59</v>
       </c>
       <c r="D24" t="n">
-        <v>0.84</v>
+        <v>0.89</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -2231,30 +2259,31 @@
       <c r="J24" t="n">
         <v>0</v>
       </c>
-      <c r="K24" s="3" t="inlineStr">
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" s="3" t="inlineStr">
         <is>
           <t>automated, app_aware</t>
         </is>
       </c>
-      <c r="L24" s="3" t="inlineStr">
+      <c r="M24" s="3" t="inlineStr">
         <is>
           <t>ua_script: 4 of 4 requests carry a script-class User-Agent; probe_paths: 1 requests for 1 scanner path families: api_docs=1</t>
         </is>
       </c>
-      <c r="M24" s="3" t="inlineStr">
+      <c r="N24" s="3" t="inlineStr">
         <is>
           <t>curl/8.7.1</t>
         </is>
       </c>
-      <c r="N24" t="n">
+      <c r="O24" t="n">
         <v>7018</v>
       </c>
-      <c r="O24" s="3" t="inlineStr">
+      <c r="P24" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P24" s="3" t="inlineStr">
+      <c r="Q24" s="3" t="inlineStr">
         <is>
           <t>1x /robots.txt [200]
 1x /.well-known/security.txt [200]
@@ -2262,7 +2291,7 @@
 1x /.well-known/openid-configuration [200]</t>
         </is>
       </c>
-      <c r="Q24" t="inlineStr">
+      <c r="R24" t="inlineStr">
         <is>
           <t>benign_user</t>
         </is>
@@ -2276,7 +2305,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="D25" t="n">
         <v>0.99</v>
@@ -2303,30 +2332,31 @@
       <c r="J25" t="n">
         <v>0</v>
       </c>
-      <c r="K25" s="3" t="inlineStr">
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr">
         <is>
           <t>automated, app_aware, declared_bot</t>
         </is>
       </c>
-      <c r="L25" s="3" t="inlineStr">
+      <c r="M25" s="3" t="inlineStr">
         <is>
           <t>ua_crawler: 30 of 30 requests carry a crawler-class User-Agent</t>
         </is>
       </c>
-      <c r="M25" s="3" t="inlineStr">
+      <c r="N25" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 (compatible; bingbot/2.0; +http://www.bing.com/bingbot.htm)</t>
         </is>
       </c>
-      <c r="N25" t="n">
+      <c r="O25" t="n">
         <v>8075</v>
       </c>
-      <c r="O25" s="3" t="inlineStr">
+      <c r="P25" s="3" t="inlineStr">
         <is>
           <t>trust.example-trust.io</t>
         </is>
       </c>
-      <c r="P25" s="3" t="inlineStr">
+      <c r="Q25" s="3" t="inlineStr">
         <is>
           <t>12x /api/v1/trust/documents [200]
 10x /acme [200]
@@ -2335,7 +2365,7 @@
 1x /acme/faq [200]</t>
         </is>
       </c>
-      <c r="Q25" t="inlineStr">
+      <c r="R25" t="inlineStr">
         <is>
           <t>benign_bot</t>
         </is>
@@ -2349,26 +2379,26 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.28</v>
+        <v>0.34</v>
       </c>
       <c r="D26" t="n">
-        <v>0.99</v>
+        <v>0.97</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>31.13.115.2</t>
+          <t>54.36.148.10</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>120</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>13:02-13:02 (0.0 min)</t>
+          <t>03:00-14:54 (714.0 min)</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I26" t="n">
         <v>0</v>
@@ -2376,100 +2406,31 @@
       <c r="J26" t="n">
         <v>0</v>
       </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t>automated, declared_bot, app_aware</t>
-        </is>
-      </c>
+      <c r="K26" t="inlineStr"/>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>ua_crawler: 2 of 2 requests carry a crawler-class User-Agent</t>
+          <t>automated, app_aware, declared_bot</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>facebookexternalhit/1.1 (+http://www.facebook.com/externalhit_uatext.php)</t>
-        </is>
-      </c>
-      <c r="N26" t="n">
-        <v>32934</v>
-      </c>
-      <c r="O26" s="3" t="inlineStr">
+          <t>ua_crawler: 120 of 120 requests carry a crawler-class User-Agent</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="inlineStr">
+        <is>
+          <t>Mozilla/5.0 (compatible; AhrefsBot/7.0; +http://ahrefs.com/robot/)</t>
+        </is>
+      </c>
+      <c r="O26" t="n">
+        <v>16276</v>
+      </c>
+      <c r="P26" s="3" t="inlineStr">
         <is>
           <t>trust.example-trust.io</t>
         </is>
       </c>
-      <c r="P26" s="3" t="inlineStr">
-        <is>
-          <t>1x /acme [200]
-1x /acme/documents [200]</t>
-        </is>
-      </c>
-      <c r="Q26" t="inlineStr">
-        <is>
-          <t>benign_bot</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr"/>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>benign_bot</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="D27" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>54.36.148.10</t>
-        </is>
-      </c>
-      <c r="F27" t="n">
-        <v>120</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>03:00-14:54 (714.0 min)</t>
-        </is>
-      </c>
-      <c r="H27" t="n">
-        <v>1</v>
-      </c>
-      <c r="I27" t="n">
-        <v>0</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0</v>
-      </c>
-      <c r="K27" s="3" t="inlineStr">
-        <is>
-          <t>automated, app_aware, declared_bot</t>
-        </is>
-      </c>
-      <c r="L27" s="3" t="inlineStr">
-        <is>
-          <t>ua_crawler: 120 of 120 requests carry a crawler-class User-Agent</t>
-        </is>
-      </c>
-      <c r="M27" s="3" t="inlineStr">
-        <is>
-          <t>Mozilla/5.0 (compatible; AhrefsBot/7.0; +http://ahrefs.com/robot/)</t>
-        </is>
-      </c>
-      <c r="N27" t="n">
-        <v>16276</v>
-      </c>
-      <c r="O27" s="3" t="inlineStr">
-        <is>
-          <t>trust.example-trust.io</t>
-        </is>
-      </c>
-      <c r="P27" s="3" t="inlineStr">
+      <c r="Q26" s="3" t="inlineStr">
         <is>
           <t>25x /acme/faq [200]
 20x /acme [200]
@@ -2480,7 +2441,78 @@
 9x /api/v1/trust/pages [200]</t>
         </is>
       </c>
-      <c r="Q27" t="inlineStr">
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>benign_bot</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+      <c r="B27" s="6" t="inlineStr">
+        <is>
+          <t>benign_bot</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>31.13.115.2</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>2</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>13:02-13:02 (0.0 min)</t>
+        </is>
+      </c>
+      <c r="H27" t="n">
+        <v>2</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0</v>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>automated, declared_bot, app_aware</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr">
+        <is>
+          <t>ua_crawler: 2 of 2 requests carry a crawler-class User-Agent</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="inlineStr">
+        <is>
+          <t>facebookexternalhit/1.1 (+http://www.facebook.com/externalhit_uatext.php)</t>
+        </is>
+      </c>
+      <c r="O27" t="n">
+        <v>32934</v>
+      </c>
+      <c r="P27" s="3" t="inlineStr">
+        <is>
+          <t>trust.example-trust.io</t>
+        </is>
+      </c>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>1x /acme [200]
+1x /acme/documents [200]</t>
+        </is>
+      </c>
+      <c r="R27" t="inlineStr">
         <is>
           <t>benign_bot</t>
         </is>
@@ -2494,7 +2526,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="D28" t="n">
         <v>0.98</v>
@@ -2521,30 +2553,31 @@
       <c r="J28" t="n">
         <v>0</v>
       </c>
-      <c r="K28" s="3" t="inlineStr">
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" s="3" t="inlineStr">
         <is>
           <t>app_aware, automated, declared_bot</t>
         </is>
       </c>
-      <c r="L28" s="3" t="inlineStr">
+      <c r="M28" s="3" t="inlineStr">
         <is>
           <t>ua_crawler: 60 of 60 requests carry a crawler-class User-Agent</t>
         </is>
       </c>
-      <c r="M28" s="3" t="inlineStr">
+      <c r="N28" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 (compatible; Googlebot/2.1; +http://www.google.com/bot.html)</t>
         </is>
       </c>
-      <c r="N28" t="n">
+      <c r="O28" t="n">
         <v>15169</v>
       </c>
-      <c r="O28" s="3" t="inlineStr">
+      <c r="P28" s="3" t="inlineStr">
         <is>
           <t>trust.example-trust.io</t>
         </is>
       </c>
-      <c r="P28" s="3" t="inlineStr">
+      <c r="Q28" s="3" t="inlineStr">
         <is>
           <t>13x /api/v1/trust/pages [200]
 11x /acme [200]
@@ -2554,7 +2587,7 @@
 7x /acme/faq [200]</t>
         </is>
       </c>
-      <c r="Q28" t="inlineStr">
+      <c r="R28" t="inlineStr">
         <is>
           <t>benign_bot</t>
         </is>
@@ -2595,35 +2628,36 @@
       <c r="J29" t="n">
         <v>0</v>
       </c>
-      <c r="K29" s="3" t="inlineStr">
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" s="3" t="inlineStr">
         <is>
           <t>automated, monitoring, declared_bot, app_aware</t>
         </is>
       </c>
-      <c r="L29" s="3" t="inlineStr">
+      <c r="M29" s="3" t="inlineStr">
         <is>
           <t>ua_monitor: 1440 of 1440 requests carry a monitor-class User-Agent</t>
         </is>
       </c>
-      <c r="M29" s="3" t="inlineStr">
+      <c r="N29" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0+(compatible; UptimeRobot/2.0; http://www.uptimerobot.com/)</t>
         </is>
       </c>
-      <c r="N29" t="n">
+      <c r="O29" t="n">
         <v>20473</v>
       </c>
-      <c r="O29" s="3" t="inlineStr">
+      <c r="P29" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P29" s="3" t="inlineStr">
+      <c r="Q29" s="3" t="inlineStr">
         <is>
           <t>1440x / [200]</t>
         </is>
       </c>
-      <c r="Q29" t="inlineStr">
+      <c r="R29" t="inlineStr">
         <is>
           <t>benign_bot</t>
         </is>
@@ -2664,35 +2698,36 @@
       <c r="J30" t="n">
         <v>0</v>
       </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t>monitoring, app_aware, automated, declared_bot</t>
-        </is>
-      </c>
+      <c r="K30" t="inlineStr"/>
       <c r="L30" s="3" t="inlineStr">
         <is>
+          <t>monitoring, automated, app_aware, declared_bot</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
           <t>ua_monitor: 288 of 288 requests carry a monitor-class User-Agent</t>
         </is>
       </c>
-      <c r="M30" s="3" t="inlineStr">
+      <c r="N30" s="3" t="inlineStr">
         <is>
           <t>Google-Cloud-Scheduler</t>
         </is>
       </c>
-      <c r="N30" t="n">
+      <c r="O30" t="n">
         <v>15169</v>
       </c>
-      <c r="O30" s="3" t="inlineStr">
+      <c r="P30" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P30" s="3" t="inlineStr">
+      <c r="Q30" s="3" t="inlineStr">
         <is>
           <t>288x /api/v1/tenant_admin/health [204]</t>
         </is>
       </c>
-      <c r="Q30" t="inlineStr">
+      <c r="R30" t="inlineStr">
         <is>
           <t>benign_bot</t>
         </is>
@@ -2706,10 +2741,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1.49</v>
+        <v>1.42</v>
       </c>
       <c r="D31" t="n">
-        <v>0.89</v>
+        <v>0.83</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -2733,30 +2768,31 @@
       <c r="J31" t="n">
         <v>0</v>
       </c>
-      <c r="K31" s="3" t="inlineStr">
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" s="3" t="inlineStr">
         <is>
           <t>app_aware, generic_probing</t>
         </is>
       </c>
-      <c r="L31" s="3" t="inlineStr">
+      <c r="M31" s="3" t="inlineStr">
         <is>
           <t>probe_paths: 1 requests for 1 scanner path families: admin_panels=1</t>
         </is>
       </c>
-      <c r="M31" s="3" t="inlineStr">
+      <c r="N31" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 (Windows NT 10.0; Win64; x64; rv:130.0) Gecko/20100101 Firefox/130.0</t>
         </is>
       </c>
-      <c r="N31" t="n">
+      <c r="O31" t="n">
         <v>3320</v>
       </c>
-      <c r="O31" s="3" t="inlineStr">
+      <c r="P31" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P31" s="3" t="inlineStr">
+      <c r="Q31" s="3" t="inlineStr">
         <is>
           <t>3x / [200]
 3x /assets/index-8f2a1c.js [200]
@@ -2768,7 +2804,7 @@
 2x /api/v1/tenants/acme/pages [200]</t>
         </is>
       </c>
-      <c r="Q31" t="inlineStr">
+      <c r="R31" t="inlineStr">
         <is>
           <t>benign_user</t>
         </is>
@@ -2782,10 +2818,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1.09</v>
+        <v>1.16</v>
       </c>
       <c r="D32" t="n">
-        <v>0.77</v>
+        <v>0.73</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -2809,26 +2845,27 @@
       <c r="J32" t="n">
         <v>0</v>
       </c>
-      <c r="K32" s="3" t="inlineStr">
+      <c r="K32" t="inlineStr"/>
+      <c r="L32" s="3" t="inlineStr">
         <is>
           <t>app_aware</t>
         </is>
       </c>
-      <c r="L32" s="3" t="inlineStr"/>
-      <c r="M32" s="3" t="inlineStr">
+      <c r="M32" s="3" t="inlineStr"/>
+      <c r="N32" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 (Macintosh; Intel Mac OS X 14_5) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/128.0.0.0 Safari/537.36</t>
         </is>
       </c>
-      <c r="N32" t="n">
+      <c r="O32" t="n">
         <v>7922</v>
       </c>
-      <c r="O32" s="3" t="inlineStr">
+      <c r="P32" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P32" s="3" t="inlineStr">
+      <c r="Q32" s="3" t="inlineStr">
         <is>
           <t>2x /api/v1/auth/mfa/verify [401/200]
 2x / [200]
@@ -2840,7 +2877,7 @@
 2x /api/v1/tenants/acme/pages [200]</t>
         </is>
       </c>
-      <c r="Q32" t="inlineStr">
+      <c r="R32" t="inlineStr">
         <is>
           <t>benign_user</t>
         </is>
@@ -2848,16 +2885,16 @@
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>unclear</t>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>benign_user</t>
         </is>
       </c>
       <c r="C33" t="n">
         <v>0.5</v>
       </c>
       <c r="D33" t="n">
-        <v>0.35</v>
+        <v>0.38</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -2881,26 +2918,27 @@
       <c r="J33" t="n">
         <v>0</v>
       </c>
-      <c r="K33" s="3" t="inlineStr">
+      <c r="K33" t="inlineStr"/>
+      <c r="L33" s="3" t="inlineStr">
         <is>
           <t>app_aware</t>
         </is>
       </c>
-      <c r="L33" s="3" t="inlineStr"/>
-      <c r="M33" s="3" t="inlineStr">
+      <c r="M33" s="3" t="inlineStr"/>
+      <c r="N33" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 (Macintosh; Intel Mac OS X 14_5) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/128.0.0.0 Safari/537.36</t>
         </is>
       </c>
-      <c r="N33" t="n">
+      <c r="O33" t="n">
         <v>7922</v>
       </c>
-      <c r="O33" s="3" t="inlineStr">
+      <c r="P33" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P33" s="3" t="inlineStr">
+      <c r="Q33" s="3" t="inlineStr">
         <is>
           <t>6x / [200]
 6x /assets/index-8f2a1c.js [200]
@@ -2912,7 +2950,7 @@
 4x /api/v1/tenants/acme/members [200]</t>
         </is>
       </c>
-      <c r="Q33" t="inlineStr">
+      <c r="R33" t="inlineStr">
         <is>
           <t>benign_user</t>
         </is>
@@ -2929,7 +2967,7 @@
         <v>0.01</v>
       </c>
       <c r="D34" t="n">
-        <v>0.55</v>
+        <v>0.57</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -2953,38 +2991,39 @@
       <c r="J34" t="n">
         <v>0</v>
       </c>
-      <c r="K34" s="3" t="inlineStr">
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" s="3" t="inlineStr">
         <is>
           <t>app_aware</t>
         </is>
       </c>
-      <c r="L34" s="3" t="inlineStr"/>
-      <c r="M34" s="3" t="inlineStr">
+      <c r="M34" s="3" t="inlineStr"/>
+      <c r="N34" s="3" t="inlineStr">
         <is>
           <t>Mozilla/5.0 (Macintosh; Intel Mac OS X 14_5) AppleWebKit/537.36 (KHTML, like Gecko) Chrome/128.0.0.0 Safari/537.36</t>
         </is>
       </c>
-      <c r="N34" t="n">
+      <c r="O34" t="n">
         <v>6939</v>
       </c>
-      <c r="O34" s="3" t="inlineStr">
+      <c r="P34" s="3" t="inlineStr">
         <is>
           <t>app.example-trust.io</t>
         </is>
       </c>
-      <c r="P34" s="3" t="inlineStr">
+      <c r="Q34" s="3" t="inlineStr">
         <is>
           <t>1x / [200]</t>
         </is>
       </c>
-      <c r="Q34" t="inlineStr">
+      <c r="R34" t="inlineStr">
         <is>
           <t>unclear</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q34"/>
+  <autoFilter ref="A1:R34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3170,7 +3209,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>2.82</v>
+        <v>2.79</v>
       </c>
       <c r="D2" t="n">
         <v>1</v>
@@ -3190,14 +3229,14 @@
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>exploit payloads against routes that exist here</t>
+          <t>exploit payloads or WAF attack signatures against routes that exist here</t>
         </is>
       </c>
       <c r="I2" t="n">
-        <v>0.82</v>
+        <v>0.79</v>
       </c>
       <c r="J2" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="K2" t="n">
         <v>0.96</v>
@@ -3209,7 +3248,7 @@
         <v>0.04</v>
       </c>
       <c r="N2" t="n">
-        <v>0.66</v>
+        <v>0.58</v>
       </c>
       <c r="O2" t="n">
         <v>0.84</v>
@@ -3227,21 +3266,21 @@
         <v>0.06</v>
       </c>
       <c r="T2" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="U2" s="3" t="inlineStr">
         <is>
-          <t>malicious 1.0, unclear 0.0, benign_bot 0.0, ai_agent 0.0, benign_user 0.0, background_scan 0.0</t>
+          <t>malicious 1.0, benign_user 0.0, unclear 0.0, ai_agent 0.0, background_scan 0.0, benign_bot 0.0</t>
         </is>
       </c>
       <c r="V2" t="n">
-        <v>4330</v>
+        <v>4433</v>
       </c>
       <c r="W2" t="n">
-        <v>2519</v>
+        <v>2572</v>
       </c>
       <c r="X2" t="n">
-        <v>316</v>
+        <v>333</v>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
@@ -3262,7 +3301,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2.78</v>
+        <v>2.79</v>
       </c>
       <c r="D3" t="n">
         <v>1</v>
@@ -3282,14 +3321,14 @@
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
-          <t>exploit payloads against routes that exist here</t>
+          <t>exploit payloads or WAF attack signatures against routes that exist here</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>0.78</v>
+        <v>0.79</v>
       </c>
       <c r="J3" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="K3" t="n">
         <v>0.96</v>
@@ -3298,7 +3337,7 @@
         <v>0.99</v>
       </c>
       <c r="M3" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="N3" t="n">
         <v>0.09</v>
@@ -3319,21 +3358,21 @@
         <v>0.04</v>
       </c>
       <c r="T3" t="n">
-        <v>0.27</v>
+        <v>0.31</v>
       </c>
       <c r="U3" s="3" t="inlineStr">
         <is>
-          <t>malicious 1.0, background_scan 0.0, benign_user 0.0, benign_bot 0.0, ai_agent 0.0, unclear 0.0</t>
+          <t>malicious 1.0, unclear 0.0, benign_user 0.0, background_scan 0.0, benign_bot 0.0, ai_agent 0.0</t>
         </is>
       </c>
       <c r="V3" t="n">
-        <v>3895</v>
+        <v>3998</v>
       </c>
       <c r="W3" t="n">
-        <v>1908</v>
+        <v>1961</v>
       </c>
       <c r="X3" t="n">
-        <v>305</v>
+        <v>319</v>
       </c>
       <c r="Y3" t="inlineStr">
         <is>
@@ -3354,7 +3393,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>2.77</v>
+        <v>2.74</v>
       </c>
       <c r="D4" t="n">
         <v>1</v>
@@ -3374,17 +3413,17 @@
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>exploit payloads against routes that exist here</t>
+          <t>exploit payloads or WAF attack signatures against routes that exist here</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>0.77</v>
+        <v>0.74</v>
       </c>
       <c r="J4" t="n">
         <v>0.05</v>
       </c>
       <c r="K4" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="L4" t="n">
         <v>0.99</v>
@@ -3399,33 +3438,33 @@
         <v>0.95</v>
       </c>
       <c r="P4" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="Q4" t="n">
         <v>0.03</v>
       </c>
       <c r="R4" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="S4" t="n">
         <v>0.04</v>
       </c>
       <c r="T4" t="n">
-        <v>0.38</v>
+        <v>0.4</v>
       </c>
       <c r="U4" s="3" t="inlineStr">
         <is>
-          <t>malicious 1.0, benign_bot 0.0, ai_agent 0.0, unclear 0.0, benign_user 0.0, background_scan 0.0</t>
+          <t>malicious 1.0, benign_bot 0.0, ai_agent 0.0, background_scan 0.0, benign_user 0.0, unclear 0.0</t>
         </is>
       </c>
       <c r="V4" t="n">
-        <v>3791</v>
+        <v>3894</v>
       </c>
       <c r="W4" t="n">
-        <v>1719</v>
+        <v>1772</v>
       </c>
       <c r="X4" t="n">
-        <v>346</v>
+        <v>382</v>
       </c>
       <c r="Y4" t="inlineStr">
         <is>
@@ -3446,7 +3485,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2.52</v>
+        <v>2.48</v>
       </c>
       <c r="D5" t="n">
         <v>0.97</v>
@@ -3470,7 +3509,7 @@
         </is>
       </c>
       <c r="I5" t="n">
-        <v>0.52</v>
+        <v>0.51</v>
       </c>
       <c r="J5" t="n">
         <v>0.04</v>
@@ -3485,7 +3524,7 @@
         <v>0.98</v>
       </c>
       <c r="N5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="O5" t="n">
         <v>0.97</v>
@@ -3507,17 +3546,17 @@
       </c>
       <c r="U5" s="3" t="inlineStr">
         <is>
-          <t>malicious 0.98, benign_bot 0.02, ai_agent 0.0, background_scan 0.0, unclear 0.0, benign_user 0.0</t>
+          <t>malicious 0.98, benign_bot 0.02, benign_user 0.0, unclear 0.0, ai_agent 0.0, background_scan 0.0</t>
         </is>
       </c>
       <c r="V5" t="n">
-        <v>3500</v>
+        <v>3604</v>
       </c>
       <c r="W5" t="n">
-        <v>1276</v>
+        <v>1330</v>
       </c>
       <c r="X5" t="n">
-        <v>818</v>
+        <v>821</v>
       </c>
       <c r="Y5" t="inlineStr">
         <is>
@@ -3538,7 +3577,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>2.34</v>
+        <v>2.32</v>
       </c>
       <c r="D6" t="n">
         <v>0.99</v>
@@ -3558,26 +3597,26 @@
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>exploit payloads against routes that exist here</t>
+          <t>exploit payloads or WAF attack signatures against routes that exist here</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>0.63</v>
+        <v>0.64</v>
       </c>
       <c r="J6" t="n">
-        <v>0.74</v>
+        <v>0.7</v>
       </c>
       <c r="K6" t="n">
         <v>0.93</v>
       </c>
       <c r="L6" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="M6" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="N6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="O6" t="n">
         <v>0.6</v>
@@ -3595,21 +3634,21 @@
         <v>0.04</v>
       </c>
       <c r="T6" t="n">
-        <v>0.22</v>
+        <v>0.26</v>
       </c>
       <c r="U6" s="3" t="inlineStr">
         <is>
-          <t>malicious 1.0, unclear 0.0, benign_user 0.0, benign_bot 0.0, ai_agent 0.0, background_scan 0.0</t>
+          <t>malicious 0.99, background_scan 0.01, unclear 0.0, benign_user 0.0, benign_bot 0.0, ai_agent 0.0</t>
         </is>
       </c>
       <c r="V6" t="n">
-        <v>3870</v>
+        <v>3973</v>
       </c>
       <c r="W6" t="n">
-        <v>1815</v>
+        <v>1869</v>
       </c>
       <c r="X6" t="n">
-        <v>318</v>
+        <v>356</v>
       </c>
       <c r="Y6" t="inlineStr">
         <is>
@@ -3630,7 +3669,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2.23</v>
+        <v>2.28</v>
       </c>
       <c r="D7" t="n">
         <v>1</v>
@@ -3650,11 +3689,11 @@
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
-          <t>exploit payloads against routes that exist here; credential attack volume with WAF or auth-volume evidence</t>
+          <t>exploit payloads or WAF attack signatures against routes that exist here; credential attack volume with WAF or auth-volume evidence</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>0.75</v>
+        <v>0.71</v>
       </c>
       <c r="J7" t="n">
         <v>0.07000000000000001</v>
@@ -3663,19 +3702,19 @@
         <v>0.95</v>
       </c>
       <c r="L7" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="M7" t="n">
-        <v>0.85</v>
+        <v>0.87</v>
       </c>
       <c r="N7" t="n">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="O7" t="n">
         <v>0.98</v>
       </c>
       <c r="P7" t="n">
-        <v>0.47</v>
+        <v>0.44</v>
       </c>
       <c r="Q7" t="n">
         <v>0.02</v>
@@ -3691,17 +3730,17 @@
       </c>
       <c r="U7" s="3" t="inlineStr">
         <is>
-          <t>malicious 1.0, benign_bot 0.0, benign_user 0.0, ai_agent 0.0, background_scan 0.0, unclear 0.0</t>
+          <t>malicious 1.0, background_scan 0.0, unclear 0.0, ai_agent 0.0, benign_user 0.0, benign_bot 0.0</t>
         </is>
       </c>
       <c r="V7" t="n">
-        <v>4077</v>
+        <v>4181</v>
       </c>
       <c r="W7" t="n">
-        <v>2106</v>
+        <v>2160</v>
       </c>
       <c r="X7" t="n">
-        <v>824</v>
+        <v>841</v>
       </c>
       <c r="Y7" t="inlineStr">
         <is>
@@ -3722,78 +3761,74 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2.18</v>
+        <v>2.15</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>0.72</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>5.188.86.2</t>
+          <t>89.248.165.2</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>420</v>
+        <v>46</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>malicious</t>
         </is>
       </c>
-      <c r="H8" s="3" t="inlineStr">
-        <is>
-          <t>credential attack volume with WAF or auth-volume evidence</t>
-        </is>
-      </c>
+      <c r="H8" s="3" t="inlineStr"/>
       <c r="I8" t="n">
-        <v>0.82</v>
+        <v>0.79</v>
       </c>
       <c r="J8" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="K8" t="n">
-        <v>0.95</v>
+        <v>0.93</v>
       </c>
       <c r="L8" t="n">
         <v>0.04</v>
       </c>
       <c r="M8" t="n">
-        <v>0.98</v>
+        <v>0.03</v>
       </c>
       <c r="N8" t="n">
-        <v>0.06</v>
+        <v>0.7</v>
       </c>
       <c r="O8" t="n">
-        <v>0.86</v>
+        <v>0.4</v>
       </c>
       <c r="P8" t="n">
         <v>0.02</v>
       </c>
       <c r="Q8" t="n">
-        <v>0.03</v>
+        <v>0.05</v>
       </c>
       <c r="R8" t="n">
         <v>0.04</v>
       </c>
       <c r="S8" t="n">
-        <v>0.04</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="T8" t="n">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="U8" s="3" t="inlineStr">
         <is>
-          <t>malicious 1.0, background_scan 0.0, benign_bot 0.0, benign_user 0.0, unclear 0.0, ai_agent 0.0</t>
+          <t>malicious 0.77, benign_user 0.15, ai_agent 0.04, benign_bot 0.04, background_scan 0.0, unclear 0.0</t>
         </is>
       </c>
       <c r="V8" t="n">
-        <v>3554</v>
+        <v>6883</v>
       </c>
       <c r="W8" t="n">
-        <v>1357</v>
+        <v>5107</v>
       </c>
       <c r="X8" t="n">
-        <v>839</v>
+        <v>406</v>
       </c>
       <c r="Y8" t="inlineStr">
         <is>
@@ -3814,74 +3849,78 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2.16</v>
+        <v>2.14</v>
       </c>
       <c r="D9" t="n">
-        <v>0.77</v>
+        <v>1</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>89.248.165.2</t>
+          <t>5.188.86.2</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>46</v>
+        <v>420</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>malicious</t>
         </is>
       </c>
-      <c r="H9" s="3" t="inlineStr"/>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>credential attack volume with WAF or auth-volume evidence</t>
+        </is>
+      </c>
       <c r="I9" t="n">
-        <v>0.79</v>
+        <v>0.86</v>
       </c>
       <c r="J9" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="K9" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="L9" t="n">
         <v>0.04</v>
       </c>
       <c r="M9" t="n">
-        <v>0.03</v>
+        <v>0.98</v>
       </c>
       <c r="N9" t="n">
-        <v>0.65</v>
+        <v>0.06</v>
       </c>
       <c r="O9" t="n">
-        <v>0.45</v>
+        <v>0.84</v>
       </c>
       <c r="P9" t="n">
         <v>0.02</v>
       </c>
       <c r="Q9" t="n">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="R9" t="n">
         <v>0.04</v>
       </c>
       <c r="S9" t="n">
-        <v>0.06</v>
+        <v>0.04</v>
       </c>
       <c r="T9" t="n">
-        <v>0.11</v>
+        <v>0.04</v>
       </c>
       <c r="U9" s="3" t="inlineStr">
         <is>
-          <t>malicious 0.81, benign_user 0.12, benign_bot 0.05, ai_agent 0.02, background_scan 0.0, unclear 0.0</t>
+          <t>malicious 1.0, background_scan 0.0, benign_bot 0.0, ai_agent 0.0, benign_user 0.0, unclear 0.0</t>
         </is>
       </c>
       <c r="V9" t="n">
-        <v>6780</v>
+        <v>3658</v>
       </c>
       <c r="W9" t="n">
-        <v>5054</v>
+        <v>1411</v>
       </c>
       <c r="X9" t="n">
-        <v>465</v>
+        <v>854</v>
       </c>
       <c r="Y9" t="inlineStr">
         <is>
@@ -3902,7 +3941,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2.09</v>
+        <v>2.12</v>
       </c>
       <c r="D10" t="n">
         <v>0.99</v>
@@ -3922,13 +3961,13 @@
       </c>
       <c r="H10" s="3" t="inlineStr"/>
       <c r="I10" t="n">
-        <v>0.89</v>
+        <v>0.86</v>
       </c>
       <c r="J10" t="n">
         <v>0.05</v>
       </c>
       <c r="K10" t="n">
-        <v>0.93</v>
+        <v>0.92</v>
       </c>
       <c r="L10" t="n">
         <v>0.04</v>
@@ -3937,7 +3976,7 @@
         <v>0.03</v>
       </c>
       <c r="N10" t="n">
-        <v>0.93</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="O10" t="n">
         <v>0.97</v>
@@ -3949,27 +3988,27 @@
         <v>0.05</v>
       </c>
       <c r="R10" t="n">
-        <v>0.11</v>
+        <v>0.09</v>
       </c>
       <c r="S10" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="T10" t="n">
-        <v>0.38</v>
+        <v>0.43</v>
       </c>
       <c r="U10" s="3" t="inlineStr">
         <is>
-          <t>malicious 0.99, benign_bot 0.01, ai_agent 0.0, benign_user 0.0, unclear 0.0, background_scan 0.0</t>
+          <t>malicious 1.0, background_scan 0.0, benign_user 0.0, ai_agent 0.0, benign_bot 0.0, unclear 0.0</t>
         </is>
       </c>
       <c r="V10" t="n">
-        <v>3598</v>
+        <v>3702</v>
       </c>
       <c r="W10" t="n">
-        <v>1391</v>
+        <v>1445</v>
       </c>
       <c r="X10" t="n">
-        <v>815</v>
+        <v>843</v>
       </c>
       <c r="Y10" t="inlineStr">
         <is>
@@ -3989,7 +4028,7 @@
         <v>1.06</v>
       </c>
       <c r="D11" t="n">
-        <v>0.78</v>
+        <v>0.8</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -4006,13 +4045,13 @@
       </c>
       <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" t="n">
-        <v>0.84</v>
+        <v>0.85</v>
       </c>
       <c r="J11" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="K11" t="n">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="L11" t="n">
         <v>0.04</v>
@@ -4024,10 +4063,10 @@
         <v>0.06</v>
       </c>
       <c r="O11" t="n">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="P11" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="Q11" t="n">
         <v>0.03</v>
@@ -4039,21 +4078,21 @@
         <v>0.97</v>
       </c>
       <c r="T11" t="n">
-        <v>0.85</v>
+        <v>0.82</v>
       </c>
       <c r="U11" s="3" t="inlineStr">
         <is>
-          <t>background_scan 0.83, unclear 0.1, benign_bot 0.04, malicious 0.03, benign_user 0.0, ai_agent 0.0</t>
+          <t>background_scan 0.84, unclear 0.09, benign_bot 0.04, malicious 0.03, benign_user 0.0, ai_agent 0.0</t>
         </is>
       </c>
       <c r="V11" t="n">
-        <v>3445</v>
+        <v>3547</v>
       </c>
       <c r="W11" t="n">
-        <v>1213</v>
+        <v>1265</v>
       </c>
       <c r="X11" t="n">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="Y11" t="inlineStr">
         <is>
@@ -4070,18 +4109,18 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1.03</v>
+        <v>1.01</v>
       </c>
       <c r="D12" t="n">
-        <v>0.5</v>
+        <v>0.95</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>87.120.104.29</t>
+          <t>80.94.95.211</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -4090,54 +4129,54 @@
       </c>
       <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" t="n">
-        <v>0.8100000000000001</v>
+        <v>0.99</v>
       </c>
       <c r="J12" t="n">
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
       <c r="K12" t="n">
-        <v>0.18</v>
+        <v>0.03</v>
       </c>
       <c r="L12" t="n">
         <v>0.04</v>
       </c>
       <c r="M12" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="N12" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="O12" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="P12" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="Q12" t="n">
         <v>0.03</v>
       </c>
-      <c r="N12" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="O12" t="n">
-        <v>0.72</v>
-      </c>
-      <c r="P12" t="n">
+      <c r="R12" t="n">
         <v>0.02</v>
       </c>
-      <c r="Q12" t="n">
-        <v>0.06</v>
-      </c>
-      <c r="R12" t="n">
-        <v>0.39</v>
-      </c>
       <c r="S12" t="n">
-        <v>0.97</v>
+        <v>0.04</v>
       </c>
       <c r="T12" t="n">
-        <v>0.05</v>
+        <v>0.98</v>
       </c>
       <c r="U12" s="3" t="inlineStr">
         <is>
-          <t>background_scan 0.59, malicious 0.12, unclear 0.11, benign_bot 0.08, benign_user 0.06, ai_agent 0.04</t>
+          <t>background_scan 0.96, malicious 0.04, benign_user 0.0, unclear 0.0, ai_agent 0.0, benign_bot 0.0</t>
         </is>
       </c>
       <c r="V12" t="n">
-        <v>3421</v>
+        <v>4518</v>
       </c>
       <c r="W12" t="n">
-        <v>1158</v>
+        <v>2560</v>
       </c>
       <c r="X12" t="n">
-        <v>442</v>
+        <v>328</v>
       </c>
       <c r="Y12" t="inlineStr">
         <is>
@@ -4154,18 +4193,18 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.01</v>
+        <v>1</v>
       </c>
       <c r="D13" t="n">
-        <v>0.96</v>
+        <v>0.45</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>80.94.95.211</t>
+          <t>87.120.104.29</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -4174,54 +4213,54 @@
       </c>
       <c r="H13" s="3" t="inlineStr"/>
       <c r="I13" t="n">
-        <v>0.99</v>
+        <v>0.8100000000000001</v>
       </c>
       <c r="J13" t="n">
-        <v>0.98</v>
+        <v>0.06</v>
       </c>
       <c r="K13" t="n">
-        <v>0.03</v>
+        <v>0.17</v>
       </c>
       <c r="L13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="Q13" t="n">
         <v>0.05</v>
       </c>
-      <c r="M13" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="N13" t="n">
-        <v>0.17</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="P13" t="n">
+      <c r="R13" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="S13" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="T13" t="n">
         <v>0.05</v>
       </c>
-      <c r="Q13" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="R13" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="S13" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="T13" t="n">
-        <v>0.98</v>
-      </c>
       <c r="U13" s="3" t="inlineStr">
         <is>
-          <t>background_scan 0.97, malicious 0.03, benign_user 0.0, ai_agent 0.0, unclear 0.0, benign_bot 0.0</t>
+          <t>background_scan 0.54, unclear 0.14, malicious 0.12, benign_bot 0.09, benign_user 0.07, ai_agent 0.04</t>
         </is>
       </c>
       <c r="V13" t="n">
-        <v>4415</v>
+        <v>3524</v>
       </c>
       <c r="W13" t="n">
-        <v>2507</v>
+        <v>1211</v>
       </c>
       <c r="X13" t="n">
-        <v>372</v>
+        <v>311</v>
       </c>
       <c r="Y13" t="inlineStr">
         <is>
@@ -4267,10 +4306,10 @@
         <v>0.03</v>
       </c>
       <c r="L14" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="M14" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="N14" t="n">
         <v>0.06</v>
@@ -4295,17 +4334,17 @@
       </c>
       <c r="U14" s="3" t="inlineStr">
         <is>
-          <t>background_scan 1.0, benign_bot 0.0, malicious 0.0, benign_user 0.0, unclear 0.0, ai_agent 0.0</t>
+          <t>background_scan 1.0, malicious 0.0, unclear 0.0, ai_agent 0.0, benign_user 0.0, benign_bot 0.0</t>
         </is>
       </c>
       <c r="V14" t="n">
-        <v>3779</v>
+        <v>3882</v>
       </c>
       <c r="W14" t="n">
-        <v>1672</v>
+        <v>1725</v>
       </c>
       <c r="X14" t="n">
-        <v>307</v>
+        <v>321</v>
       </c>
       <c r="Y14" t="inlineStr">
         <is>
@@ -4348,7 +4387,7 @@
         <v>0.98</v>
       </c>
       <c r="K15" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="L15" t="n">
         <v>0.04</v>
@@ -4360,7 +4399,7 @@
         <v>0.08</v>
       </c>
       <c r="O15" t="n">
-        <v>0.89</v>
+        <v>0.87</v>
       </c>
       <c r="P15" t="n">
         <v>0.02</v>
@@ -4372,24 +4411,24 @@
         <v>0.03</v>
       </c>
       <c r="S15" t="n">
-        <v>0.97</v>
+        <v>0.98</v>
       </c>
       <c r="T15" t="n">
-        <v>0.82</v>
+        <v>0.78</v>
       </c>
       <c r="U15" s="3" t="inlineStr">
         <is>
-          <t>background_scan 1.0, benign_bot 0.0, malicious 0.0, benign_user 0.0, unclear 0.0, ai_agent 0.0</t>
+          <t>background_scan 1.0, benign_user 0.0, ai_agent 0.0, unclear 0.0, benign_bot 0.0, malicious 0.0</t>
         </is>
       </c>
       <c r="V15" t="n">
-        <v>3855</v>
+        <v>3958</v>
       </c>
       <c r="W15" t="n">
-        <v>1799</v>
+        <v>1853</v>
       </c>
       <c r="X15" t="n">
-        <v>334</v>
+        <v>340</v>
       </c>
       <c r="Y15" t="inlineStr">
         <is>
@@ -4435,7 +4474,7 @@
         <v>0.02</v>
       </c>
       <c r="L16" t="n">
-        <v>0.48</v>
+        <v>0.29</v>
       </c>
       <c r="M16" t="n">
         <v>0.03</v>
@@ -4450,7 +4489,7 @@
         <v>0.02</v>
       </c>
       <c r="Q16" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="R16" t="n">
         <v>0.03</v>
@@ -4459,21 +4498,21 @@
         <v>0.98</v>
       </c>
       <c r="T16" t="n">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="U16" s="3" t="inlineStr">
         <is>
-          <t>background_scan 1.0, benign_user 0.0, malicious 0.0, unclear 0.0, benign_bot 0.0, ai_agent 0.0</t>
+          <t>background_scan 1.0, malicious 0.0, unclear 0.0, benign_user 0.0, benign_bot 0.0, ai_agent 0.0</t>
         </is>
       </c>
       <c r="V16" t="n">
-        <v>3697</v>
+        <v>3799</v>
       </c>
       <c r="W16" t="n">
-        <v>1575</v>
+        <v>1627</v>
       </c>
       <c r="X16" t="n">
-        <v>283</v>
+        <v>327</v>
       </c>
       <c r="Y16" t="inlineStr">
         <is>
@@ -4490,10 +4529,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.49</v>
       </c>
       <c r="D17" t="n">
-        <v>0.82</v>
+        <v>0.85</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -4510,10 +4549,10 @@
       </c>
       <c r="H17" s="3" t="inlineStr"/>
       <c r="I17" t="n">
-        <v>0.44</v>
+        <v>0.51</v>
       </c>
       <c r="J17" t="n">
-        <v>0.17</v>
+        <v>0.18</v>
       </c>
       <c r="K17" t="n">
         <v>0.21</v>
@@ -4543,21 +4582,21 @@
         <v>0.97</v>
       </c>
       <c r="T17" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="U17" s="3" t="inlineStr">
         <is>
-          <t>background_scan 0.85, benign_bot 0.09, unclear 0.03, ai_agent 0.02, malicious 0.01, benign_user 0.0</t>
+          <t>background_scan 0.88, benign_bot 0.09, unclear 0.02, ai_agent 0.01, malicious 0.0, benign_user 0.0</t>
         </is>
       </c>
       <c r="V17" t="n">
-        <v>3502</v>
+        <v>3604</v>
       </c>
       <c r="W17" t="n">
-        <v>1302</v>
+        <v>1355</v>
       </c>
       <c r="X17" t="n">
-        <v>320</v>
+        <v>331</v>
       </c>
       <c r="Y17" t="inlineStr">
         <is>
@@ -4574,10 +4613,10 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.7</v>
+        <v>0.74</v>
       </c>
       <c r="D18" t="n">
-        <v>1</v>
+        <v>0.99</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -4594,54 +4633,54 @@
       </c>
       <c r="H18" s="3" t="inlineStr"/>
       <c r="I18" t="n">
-        <v>0.44</v>
+        <v>0.45</v>
       </c>
       <c r="J18" t="n">
         <v>0.04</v>
       </c>
       <c r="K18" t="n">
-        <v>0.92</v>
+        <v>0.91</v>
       </c>
       <c r="L18" t="n">
         <v>0.04</v>
       </c>
       <c r="M18" t="n">
-        <v>0.02</v>
+        <v>0.03</v>
       </c>
       <c r="N18" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="O18" t="n">
-        <v>0.86</v>
+        <v>0.85</v>
       </c>
       <c r="P18" t="n">
-        <v>0.29</v>
+        <v>0.26</v>
       </c>
       <c r="Q18" t="n">
         <v>0.98</v>
       </c>
       <c r="R18" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="S18" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="T18" t="n">
         <v>0.03</v>
       </c>
       <c r="U18" s="3" t="inlineStr">
         <is>
-          <t>ai_agent 1.0, benign_user 0.0, unclear 0.0, background_scan 0.0, benign_bot 0.0, malicious 0.0</t>
+          <t>ai_agent 0.99, benign_bot 0.01, benign_user 0.0, unclear 0.0, background_scan 0.0, malicious 0.0</t>
         </is>
       </c>
       <c r="V18" t="n">
-        <v>3595</v>
+        <v>3697</v>
       </c>
       <c r="W18" t="n">
-        <v>1403</v>
+        <v>1455</v>
       </c>
       <c r="X18" t="n">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="Y18" t="inlineStr">
         <is>
@@ -4658,7 +4697,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.64</v>
+        <v>0.71</v>
       </c>
       <c r="D19" t="n">
         <v>1</v>
@@ -4678,7 +4717,7 @@
       </c>
       <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" t="n">
-        <v>0.36</v>
+        <v>0.29</v>
       </c>
       <c r="J19" t="n">
         <v>0.04</v>
@@ -4690,19 +4729,19 @@
         <v>0.04</v>
       </c>
       <c r="M19" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="N19" t="n">
         <v>0.06</v>
       </c>
       <c r="O19" t="n">
-        <v>0.9</v>
+        <v>0.91</v>
       </c>
       <c r="P19" t="n">
-        <v>0.63</v>
+        <v>0.68</v>
       </c>
       <c r="Q19" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="R19" t="n">
         <v>0.08</v>
@@ -4715,17 +4754,17 @@
       </c>
       <c r="U19" s="3" t="inlineStr">
         <is>
-          <t>ai_agent 1.0, benign_bot 0.0, benign_user 0.0, unclear 0.0, malicious 0.0, background_scan 0.0</t>
+          <t>ai_agent 1.0, benign_user 0.0, benign_bot 0.0, unclear 0.0, malicious 0.0, background_scan 0.0</t>
         </is>
       </c>
       <c r="V19" t="n">
-        <v>3637</v>
+        <v>3740</v>
       </c>
       <c r="W19" t="n">
-        <v>1475</v>
+        <v>1528</v>
       </c>
       <c r="X19" t="n">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="Y19" t="inlineStr">
         <is>
@@ -4742,18 +4781,18 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.58</v>
+        <v>0.49</v>
       </c>
       <c r="D20" t="n">
-        <v>0.99</v>
+        <v>0.98</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>3.15.8.8</t>
+          <t>20.171.207.1</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>25</v>
+        <v>80</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -4762,7 +4801,7 @@
       </c>
       <c r="H20" s="3" t="inlineStr"/>
       <c r="I20" t="n">
-        <v>0.42</v>
+        <v>0.51</v>
       </c>
       <c r="J20" t="n">
         <v>0.04</v>
@@ -4771,7 +4810,7 @@
         <v>0.96</v>
       </c>
       <c r="L20" t="n">
-        <v>0.03</v>
+        <v>0.04</v>
       </c>
       <c r="M20" t="n">
         <v>0.02</v>
@@ -4780,16 +4819,16 @@
         <v>0.08</v>
       </c>
       <c r="O20" t="n">
-        <v>0.96</v>
+        <v>0.93</v>
       </c>
       <c r="P20" t="n">
-        <v>0.9</v>
+        <v>0.92</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="R20" t="n">
-        <v>0.24</v>
+        <v>0.09</v>
       </c>
       <c r="S20" t="n">
         <v>0.04</v>
@@ -4799,17 +4838,17 @@
       </c>
       <c r="U20" s="3" t="inlineStr">
         <is>
-          <t>ai_agent 0.99, benign_bot 0.01, benign_user 0.0, malicious 0.0, unclear 0.0, background_scan 0.0</t>
+          <t>ai_agent 0.98, benign_bot 0.02, benign_user 0.0, unclear 0.0, background_scan 0.0, malicious 0.0</t>
         </is>
       </c>
       <c r="V20" t="n">
-        <v>3608</v>
+        <v>3779</v>
       </c>
       <c r="W20" t="n">
-        <v>1434</v>
+        <v>1554</v>
       </c>
       <c r="X20" t="n">
-        <v>298</v>
+        <v>285</v>
       </c>
       <c r="Y20" t="inlineStr">
         <is>
@@ -4826,18 +4865,18 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.51</v>
+        <v>0.48</v>
       </c>
       <c r="D21" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>20.171.207.1</t>
+          <t>3.15.8.8</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>80</v>
+        <v>25</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -4846,7 +4885,7 @@
       </c>
       <c r="H21" s="3" t="inlineStr"/>
       <c r="I21" t="n">
-        <v>0.49</v>
+        <v>0.52</v>
       </c>
       <c r="J21" t="n">
         <v>0.04</v>
@@ -4858,13 +4897,13 @@
         <v>0.03</v>
       </c>
       <c r="M21" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="N21" t="n">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="O21" t="n">
-        <v>0.93</v>
+        <v>0.95</v>
       </c>
       <c r="P21" t="n">
         <v>0.91</v>
@@ -4873,27 +4912,27 @@
         <v>0.98</v>
       </c>
       <c r="R21" t="n">
-        <v>0.08</v>
+        <v>0.22</v>
       </c>
       <c r="S21" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="T21" t="n">
         <v>0.02</v>
       </c>
       <c r="U21" s="3" t="inlineStr">
         <is>
-          <t>ai_agent 0.99, benign_bot 0.01, benign_user 0.0, malicious 0.0, background_scan 0.0, unclear 0.0</t>
+          <t>ai_agent 0.99, benign_bot 0.01, background_scan 0.0, benign_user 0.0, malicious 0.0, unclear 0.0</t>
         </is>
       </c>
       <c r="V21" t="n">
-        <v>3676</v>
+        <v>3711</v>
       </c>
       <c r="W21" t="n">
-        <v>1501</v>
+        <v>1487</v>
       </c>
       <c r="X21" t="n">
-        <v>295</v>
+        <v>317</v>
       </c>
       <c r="Y21" t="inlineStr">
         <is>
@@ -4910,7 +4949,7 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.37</v>
+        <v>0.4</v>
       </c>
       <c r="D22" t="n">
         <v>0.99</v>
@@ -4930,31 +4969,31 @@
       </c>
       <c r="H22" s="3" t="inlineStr"/>
       <c r="I22" t="n">
-        <v>0.63</v>
+        <v>0.6</v>
       </c>
       <c r="J22" t="n">
         <v>0.04</v>
       </c>
       <c r="K22" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="L22" t="n">
         <v>0.03</v>
       </c>
       <c r="M22" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="N22" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="O22" t="n">
-        <v>0.92</v>
+        <v>0.91</v>
       </c>
       <c r="P22" t="n">
         <v>0.9</v>
       </c>
       <c r="Q22" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="R22" t="n">
         <v>0.1</v>
@@ -4971,13 +5010,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>3667</v>
+        <v>3770</v>
       </c>
       <c r="W22" t="n">
-        <v>1494</v>
+        <v>1547</v>
       </c>
       <c r="X22" t="n">
-        <v>334</v>
+        <v>304</v>
       </c>
       <c r="Y22" t="inlineStr">
         <is>
@@ -4994,10 +5033,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.92</v>
+        <v>0.71</v>
       </c>
       <c r="D23" t="n">
-        <v>0.98</v>
+        <v>0.99</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -5014,7 +5053,7 @@
       </c>
       <c r="H23" s="3" t="inlineStr"/>
       <c r="I23" t="n">
-        <v>0.08</v>
+        <v>0.29</v>
       </c>
       <c r="J23" t="n">
         <v>0.04</v>
@@ -5026,22 +5065,22 @@
         <v>0.03</v>
       </c>
       <c r="M23" t="n">
-        <v>0.03</v>
+        <v>0.02</v>
       </c>
       <c r="N23" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="O23" t="n">
-        <v>0.96</v>
+        <v>0.97</v>
       </c>
       <c r="P23" t="n">
         <v>0.06</v>
       </c>
       <c r="Q23" t="n">
-        <v>0.06</v>
+        <v>0.05</v>
       </c>
       <c r="R23" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.65</v>
       </c>
       <c r="S23" t="n">
         <v>0.04</v>
@@ -5051,17 +5090,17 @@
       </c>
       <c r="U23" s="3" t="inlineStr">
         <is>
-          <t>benign_bot 0.99, malicious 0.01, unclear 0.0, benign_user 0.0, background_scan 0.0, ai_agent 0.0</t>
+          <t>benign_bot 0.99, malicious 0.01, unclear 0.0, background_scan 0.0, benign_user 0.0, ai_agent 0.0</t>
         </is>
       </c>
       <c r="V23" t="n">
-        <v>3397</v>
+        <v>3500</v>
       </c>
       <c r="W23" t="n">
-        <v>1153</v>
+        <v>1206</v>
       </c>
       <c r="X23" t="n">
-        <v>881</v>
+        <v>854</v>
       </c>
       <c r="Y23" t="inlineStr">
         <is>
@@ -5078,10 +5117,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.65</v>
+        <v>0.59</v>
       </c>
       <c r="D24" t="n">
-        <v>0.84</v>
+        <v>0.89</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -5098,13 +5137,13 @@
       </c>
       <c r="H24" s="3" t="inlineStr"/>
       <c r="I24" t="n">
-        <v>0.35</v>
+        <v>0.41</v>
       </c>
       <c r="J24" t="n">
         <v>0.12</v>
       </c>
       <c r="K24" t="n">
-        <v>0.51</v>
+        <v>0.52</v>
       </c>
       <c r="L24" t="n">
         <v>0.04</v>
@@ -5125,27 +5164,27 @@
         <v>0.06</v>
       </c>
       <c r="R24" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="S24" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="T24" t="n">
         <v>0.12</v>
       </c>
-      <c r="S24" t="n">
-        <v>0.04</v>
-      </c>
-      <c r="T24" t="n">
-        <v>0.13</v>
-      </c>
       <c r="U24" s="3" t="inlineStr">
         <is>
-          <t>benign_bot 0.88, ai_agent 0.07, background_scan 0.04, unclear 0.01, benign_user 0.0, malicious 0.0</t>
+          <t>benign_bot 0.92, ai_agent 0.05, background_scan 0.02, unclear 0.01, benign_user 0.0, malicious 0.0</t>
         </is>
       </c>
       <c r="V24" t="n">
-        <v>3496</v>
+        <v>3598</v>
       </c>
       <c r="W24" t="n">
-        <v>1323</v>
+        <v>1375</v>
       </c>
       <c r="X24" t="n">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="Y24" t="inlineStr">
         <is>
@@ -5162,7 +5201,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.34</v>
+        <v>0.36</v>
       </c>
       <c r="D25" t="n">
         <v>0.99</v>
@@ -5182,7 +5221,7 @@
       </c>
       <c r="H25" s="3" t="inlineStr"/>
       <c r="I25" t="n">
-        <v>0.66</v>
+        <v>0.64</v>
       </c>
       <c r="J25" t="n">
         <v>0.04</v>
@@ -5197,19 +5236,19 @@
         <v>0.02</v>
       </c>
       <c r="N25" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="O25" t="n">
         <v>0.97</v>
       </c>
       <c r="P25" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.93</v>
       </c>
       <c r="Q25" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="R25" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="S25" t="n">
         <v>0.04</v>
@@ -5219,17 +5258,17 @@
       </c>
       <c r="U25" s="3" t="inlineStr">
         <is>
-          <t>benign_bot 0.99, ai_agent 0.01, background_scan 0.0, benign_user 0.0, malicious 0.0, unclear 0.0</t>
+          <t>benign_bot 0.99, ai_agent 0.01, benign_user 0.0, background_scan 0.0, unclear 0.0, malicious 0.0</t>
         </is>
       </c>
       <c r="V25" t="n">
-        <v>3653</v>
+        <v>3756</v>
       </c>
       <c r="W25" t="n">
-        <v>1470</v>
+        <v>1523</v>
       </c>
       <c r="X25" t="n">
-        <v>299</v>
+        <v>391</v>
       </c>
       <c r="Y25" t="inlineStr">
         <is>
@@ -5246,18 +5285,18 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>0.28</v>
+        <v>0.34</v>
       </c>
       <c r="D26" t="n">
-        <v>0.99</v>
+        <v>0.97</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>31.13.115.2</t>
+          <t>54.36.148.10</t>
         </is>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>120</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -5266,54 +5305,54 @@
       </c>
       <c r="H26" s="3" t="inlineStr"/>
       <c r="I26" t="n">
-        <v>0.72</v>
+        <v>0.66</v>
       </c>
       <c r="J26" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="K26" t="n">
-        <v>0.89</v>
+        <v>0.96</v>
       </c>
       <c r="L26" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="M26" t="n">
         <v>0.02</v>
       </c>
       <c r="N26" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="O26" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="P26" t="n">
+        <v>0.93</v>
+      </c>
+      <c r="Q26" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="O26" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="P26" t="n">
-        <v>0.91</v>
-      </c>
-      <c r="Q26" t="n">
-        <v>0.1</v>
-      </c>
       <c r="R26" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="S26" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="T26" t="n">
         <v>0.03</v>
       </c>
       <c r="U26" s="3" t="inlineStr">
         <is>
-          <t>benign_bot 1.0, unclear 0.0, malicious 0.0, ai_agent 0.0, benign_user 0.0, background_scan 0.0</t>
+          <t>benign_bot 0.97, ai_agent 0.02, malicious 0.01, benign_user 0.0, unclear 0.0, background_scan 0.0</t>
         </is>
       </c>
       <c r="V26" t="n">
-        <v>3429</v>
+        <v>3907</v>
       </c>
       <c r="W26" t="n">
-        <v>1214</v>
+        <v>1701</v>
       </c>
       <c r="X26" t="n">
-        <v>360</v>
+        <v>893</v>
       </c>
       <c r="Y26" t="inlineStr">
         <is>
@@ -5330,18 +5369,18 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>0.24</v>
+        <v>0.3</v>
       </c>
       <c r="D27" t="n">
-        <v>0.97</v>
+        <v>0.99</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>54.36.148.10</t>
+          <t>31.13.115.2</t>
         </is>
       </c>
       <c r="F27" t="n">
-        <v>120</v>
+        <v>2</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -5350,54 +5389,54 @@
       </c>
       <c r="H27" s="3" t="inlineStr"/>
       <c r="I27" t="n">
-        <v>0.76</v>
+        <v>0.7</v>
       </c>
       <c r="J27" t="n">
         <v>0.04</v>
       </c>
       <c r="K27" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L27" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="M27" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N27" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="O27" t="n">
         <v>0.96</v>
       </c>
-      <c r="L27" t="n">
-        <v>0.03</v>
-      </c>
-      <c r="M27" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="N27" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="O27" t="n">
-        <v>0.98</v>
-      </c>
       <c r="P27" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.91</v>
       </c>
       <c r="Q27" t="n">
         <v>0.07000000000000001</v>
       </c>
       <c r="R27" t="n">
-        <v>0.12</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="S27" t="n">
         <v>0.05</v>
       </c>
       <c r="T27" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="U27" s="3" t="inlineStr">
         <is>
-          <t>benign_bot 0.98, ai_agent 0.02, benign_user 0.0, unclear 0.0, malicious 0.0, background_scan 0.0</t>
+          <t>benign_bot 1.0, background_scan 0.0, benign_user 0.0, ai_agent 0.0, malicious 0.0, unclear 0.0</t>
         </is>
       </c>
       <c r="V27" t="n">
-        <v>3803</v>
+        <v>3531</v>
       </c>
       <c r="W27" t="n">
-        <v>1647</v>
+        <v>1267</v>
       </c>
       <c r="X27" t="n">
-        <v>788</v>
+        <v>370</v>
       </c>
       <c r="Y27" t="inlineStr">
         <is>
@@ -5414,7 +5453,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="D28" t="n">
         <v>0.98</v>
@@ -5434,13 +5473,13 @@
       </c>
       <c r="H28" s="3" t="inlineStr"/>
       <c r="I28" t="n">
-        <v>0.88</v>
+        <v>0.87</v>
       </c>
       <c r="J28" t="n">
         <v>0.04</v>
       </c>
       <c r="K28" t="n">
-        <v>0.96</v>
+        <v>0.95</v>
       </c>
       <c r="L28" t="n">
         <v>0.03</v>
@@ -5458,7 +5497,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="Q28" t="n">
-        <v>0.17</v>
+        <v>0.11</v>
       </c>
       <c r="R28" t="n">
         <v>0.06</v>
@@ -5471,17 +5510,17 @@
       </c>
       <c r="U28" s="3" t="inlineStr">
         <is>
-          <t>benign_bot 0.98, ai_agent 0.02, benign_user 0.0, unclear 0.0, malicious 0.0, background_scan 0.0</t>
+          <t>benign_bot 0.99, ai_agent 0.01, unclear 0.0, background_scan 0.0, benign_user 0.0, malicious 0.0</t>
         </is>
       </c>
       <c r="V28" t="n">
-        <v>3695</v>
+        <v>3798</v>
       </c>
       <c r="W28" t="n">
-        <v>1519</v>
+        <v>1572</v>
       </c>
       <c r="X28" t="n">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="Y28" t="inlineStr">
         <is>
@@ -5521,10 +5560,10 @@
         <v>1</v>
       </c>
       <c r="J29" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="K29" t="n">
-        <v>0.55</v>
+        <v>0.53</v>
       </c>
       <c r="L29" t="n">
         <v>0.03</v>
@@ -5548,24 +5587,24 @@
         <v>0.97</v>
       </c>
       <c r="S29" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="T29" t="n">
         <v>0.02</v>
       </c>
       <c r="U29" s="3" t="inlineStr">
         <is>
-          <t>benign_bot 1.0, background_scan 0.0, benign_user 0.0, malicious 0.0, ai_agent 0.0, unclear 0.0</t>
+          <t>benign_bot 1.0, malicious 0.0, background_scan 0.0, unclear 0.0, ai_agent 0.0, benign_user 0.0</t>
         </is>
       </c>
       <c r="V29" t="n">
-        <v>3430</v>
+        <v>3535</v>
       </c>
       <c r="W29" t="n">
-        <v>1177</v>
+        <v>1231</v>
       </c>
       <c r="X29" t="n">
-        <v>924</v>
+        <v>880</v>
       </c>
       <c r="Y29" t="inlineStr">
         <is>
@@ -5605,10 +5644,10 @@
         <v>1</v>
       </c>
       <c r="J30" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="K30" t="n">
-        <v>0.98</v>
+        <v>0.97</v>
       </c>
       <c r="L30" t="n">
         <v>0.03</v>
@@ -5626,7 +5665,7 @@
         <v>0.9399999999999999</v>
       </c>
       <c r="Q30" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="R30" t="n">
         <v>0.99</v>
@@ -5639,17 +5678,17 @@
       </c>
       <c r="U30" s="3" t="inlineStr">
         <is>
-          <t>benign_bot 1.0, benign_user 0.0, unclear 0.0, ai_agent 0.0, malicious 0.0, background_scan 0.0</t>
+          <t>benign_bot 1.0, benign_user 0.0, malicious 0.0, background_scan 0.0, ai_agent 0.0, unclear 0.0</t>
         </is>
       </c>
       <c r="V30" t="n">
-        <v>3375</v>
+        <v>3479</v>
       </c>
       <c r="W30" t="n">
-        <v>1120</v>
+        <v>1174</v>
       </c>
       <c r="X30" t="n">
-        <v>787</v>
+        <v>868</v>
       </c>
       <c r="Y30" t="inlineStr">
         <is>
@@ -5666,10 +5705,10 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1.49</v>
+        <v>1.42</v>
       </c>
       <c r="D31" t="n">
-        <v>0.89</v>
+        <v>0.83</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -5686,10 +5725,10 @@
       </c>
       <c r="H31" s="3" t="inlineStr"/>
       <c r="I31" t="n">
-        <v>0.32</v>
+        <v>0.29</v>
       </c>
       <c r="J31" t="n">
-        <v>0.67</v>
+        <v>0.71</v>
       </c>
       <c r="K31" t="n">
         <v>0.93</v>
@@ -5698,13 +5737,13 @@
         <v>0.04</v>
       </c>
       <c r="M31" t="n">
-        <v>0.04</v>
+        <v>0.05</v>
       </c>
       <c r="N31" t="n">
         <v>0.08</v>
       </c>
       <c r="O31" t="n">
-        <v>0.27</v>
+        <v>0.28</v>
       </c>
       <c r="P31" t="n">
         <v>0.02</v>
@@ -5713,7 +5752,7 @@
         <v>0.04</v>
       </c>
       <c r="R31" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="S31" t="n">
         <v>0.04</v>
@@ -5723,17 +5762,17 @@
       </c>
       <c r="U31" s="3" t="inlineStr">
         <is>
-          <t>benign_user 0.91, benign_bot 0.04, malicious 0.03, ai_agent 0.02, unclear 0.0, background_scan 0.0</t>
+          <t>benign_user 0.86, benign_bot 0.07, malicious 0.04, ai_agent 0.03, unclear 0.0, background_scan 0.0</t>
         </is>
       </c>
       <c r="V31" t="n">
-        <v>4192</v>
+        <v>4295</v>
       </c>
       <c r="W31" t="n">
-        <v>2167</v>
+        <v>2220</v>
       </c>
       <c r="X31" t="n">
-        <v>298</v>
+        <v>357</v>
       </c>
       <c r="Y31" t="inlineStr">
         <is>
@@ -5750,10 +5789,10 @@
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1.09</v>
+        <v>1.16</v>
       </c>
       <c r="D32" t="n">
-        <v>0.77</v>
+        <v>0.73</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -5788,7 +5827,7 @@
         <v>0.06</v>
       </c>
       <c r="O32" t="n">
-        <v>0.33</v>
+        <v>0.34</v>
       </c>
       <c r="P32" t="n">
         <v>0.02</v>
@@ -5807,17 +5846,17 @@
       </c>
       <c r="U32" s="3" t="inlineStr">
         <is>
-          <t>benign_user 0.8, benign_bot 0.09, ai_agent 0.06, malicious 0.05, unclear 0.0, background_scan 0.0</t>
+          <t>benign_user 0.78, benign_bot 0.1, ai_agent 0.07, malicious 0.05, background_scan 0.0, unclear 0.0</t>
         </is>
       </c>
       <c r="V32" t="n">
-        <v>4075</v>
+        <v>4178</v>
       </c>
       <c r="W32" t="n">
-        <v>1997</v>
+        <v>2050</v>
       </c>
       <c r="X32" t="n">
-        <v>342</v>
+        <v>316</v>
       </c>
       <c r="Y32" t="inlineStr">
         <is>
@@ -5828,16 +5867,16 @@
     </row>
     <row r="33">
       <c r="A33" t="inlineStr"/>
-      <c r="B33" s="8" t="inlineStr">
-        <is>
-          <t>unclear</t>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>benign_user</t>
         </is>
       </c>
       <c r="C33" t="n">
         <v>0.5</v>
       </c>
       <c r="D33" t="n">
-        <v>0.35</v>
+        <v>0.38</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -5849,12 +5888,12 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>benign_bot</t>
+          <t>benign_user</t>
         </is>
       </c>
       <c r="H33" s="3" t="inlineStr">
         <is>
-          <t>choice confidence 0.35 below 0.45</t>
+          <t>low choice confidence 0.38 but harmless either way (0.91)</t>
         </is>
       </c>
       <c r="I33" t="n">
@@ -5867,7 +5906,7 @@
         <v>0.97</v>
       </c>
       <c r="L33" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="M33" t="n">
         <v>0.05</v>
@@ -5888,24 +5927,24 @@
         <v>0.06</v>
       </c>
       <c r="S33" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="T33" t="n">
         <v>0.02</v>
       </c>
       <c r="U33" s="3" t="inlineStr">
         <is>
-          <t>benign_bot 0.46, benign_user 0.46, ai_agent 0.07, malicious 0.01, unclear 0.0, background_scan 0.0</t>
+          <t>benign_user 0.49, benign_bot 0.42, ai_agent 0.08, malicious 0.01, background_scan 0.0, unclear 0.0</t>
         </is>
       </c>
       <c r="V33" t="n">
-        <v>4040</v>
+        <v>4143</v>
       </c>
       <c r="W33" t="n">
-        <v>1944</v>
+        <v>1997</v>
       </c>
       <c r="X33" t="n">
-        <v>301</v>
+        <v>400</v>
       </c>
       <c r="Y33" t="inlineStr">
         <is>
@@ -5925,7 +5964,7 @@
         <v>0.01</v>
       </c>
       <c r="D34" t="n">
-        <v>0.55</v>
+        <v>0.57</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -5952,10 +5991,10 @@
         <v>0.05</v>
       </c>
       <c r="K34" t="n">
-        <v>0.62</v>
+        <v>0.54</v>
       </c>
       <c r="L34" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="M34" t="n">
         <v>0.02</v>
@@ -5964,7 +6003,7 @@
         <v>0.05</v>
       </c>
       <c r="O34" t="n">
-        <v>0.25</v>
+        <v>0.24</v>
       </c>
       <c r="P34" t="n">
         <v>0.02</v>
@@ -5976,24 +6015,24 @@
         <v>0.06</v>
       </c>
       <c r="S34" t="n">
-        <v>0.04</v>
+        <v>0.03</v>
       </c>
       <c r="T34" t="n">
         <v>0.02</v>
       </c>
       <c r="U34" s="3" t="inlineStr">
         <is>
-          <t>benign_user 0.63, unclear 0.36, benign_bot 0.01, malicious 0.0, ai_agent 0.0, background_scan 0.0</t>
+          <t>benign_user 0.64, unclear 0.35, benign_bot 0.01, ai_agent 0.0, background_scan 0.0, malicious 0.0</t>
         </is>
       </c>
       <c r="V34" t="n">
-        <v>3361</v>
+        <v>3463</v>
       </c>
       <c r="W34" t="n">
-        <v>1075</v>
+        <v>1127</v>
       </c>
       <c r="X34" t="n">
-        <v>275</v>
+        <v>318</v>
       </c>
       <c r="Y34" t="inlineStr">
         <is>
@@ -6118,7 +6157,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -6128,7 +6167,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -6148,7 +6187,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>125638</v>
+        <v>129038</v>
       </c>
     </row>
     <row r="13">
@@ -6158,7 +6197,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>3667</v>
+        <v>3770</v>
       </c>
     </row>
     <row r="14">
@@ -6168,7 +6207,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>6780</v>
+        <v>6883</v>
       </c>
     </row>
     <row r="15">
@@ -6178,7 +6217,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0.1599</v>
+        <v>0.1642</v>
       </c>
     </row>
     <row r="16">
@@ -6188,7 +6227,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>334</v>
+        <v>340</v>
       </c>
     </row>
     <row r="17">
@@ -6256,7 +6295,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>{'host': 3689, 'query': 648, 'ua': 3682, 'referer': 93, 'waf_action': 3689, 'waf_rule': 506, 'asn': 3689, 'country': 0, 'ja3': 0, 'ja4': 0, 'bytes_in': 0, 'bytes_out': 0, 'latency_ms': 0, 'protocol': 0, 'target': 0, 'source': 3689}</t>
+          <t>{'status': 3689, 'host': 3689, 'query': 648, 'ua': 3682, 'referer': 93, 'waf_action': 3689, 'waf_rule': 506, 'waf_labels': 0, 'asn': 3689, 'country': 0, 'ja3': 0, 'ja4': 0, 'bytes_in': 0, 'bytes_out': 0, 'latency_ms': 0, 'protocol': 0, 'target': 0, 'source': 3689}</t>
         </is>
       </c>
     </row>
@@ -6292,7 +6331,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.97</v>
       </c>
     </row>
     <row r="26">
@@ -6303,7 +6342,7 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>{'benign_user': {'labelled': 4, 'predicted': 2, 'correct': 2, 'recall': 0.5, 'precision': 1.0}, 'benign_bot': {'labelled': 7, 'predicted': 8, 'correct': 7, 'recall': 1.0, 'precision': 0.88}, 'ai_agent': {'labelled': 5, 'predicted': 5, 'correct': 5, 'recall': 1.0, 'precision': 1.0}, 'background_scan': {'labelled': 7, 'predicted': 7, 'correct': 7, 'recall': 1.0, 'precision': 1.0}, 'malicious': {'labelled': 9, 'predicted': 9, 'correct': 9, 'recall': 1.0, 'precision': 1.0}, 'unclear': {'labelled': 1, 'predicted': 2, 'correct': 1, 'recall': 1.0, 'precision': 0.5}}</t>
+          <t>{'benign_user': {'labelled': 4, 'predicted': 3, 'correct': 3, 'recall': 0.75, 'precision': 1.0}, 'benign_bot': {'labelled': 7, 'predicted': 8, 'correct': 7, 'recall': 1.0, 'precision': 0.88}, 'ai_agent': {'labelled': 5, 'predicted': 5, 'correct': 5, 'recall': 1.0, 'precision': 1.0}, 'background_scan': {'labelled': 7, 'predicted': 7, 'correct': 7, 'recall': 1.0, 'precision': 1.0}, 'malicious': {'labelled': 9, 'predicted': 9, 'correct': 9, 'recall': 1.0, 'precision': 1.0}, 'unclear': {'labelled': 1, 'predicted': 1, 'correct': 1, 'recall': 1.0, 'precision': 1.0}}</t>
         </is>
       </c>
     </row>

</xml_diff>